<commit_message>
Add October work hours to production log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ugCjvyp7meZnJb6nyvem6
</commit_message>
<xml_diff>
--- a/מעקב הפקה - אוקטובר נובמבר 2026.xlsx
+++ b/מעקב הפקה - אוקטובר נובמבר 2026.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="[$-40D]ddd dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-40D]ddd dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <charset val="177"/>
@@ -72,6 +72,15 @@
       <name val="Arial"/>
       <family val="2"/>
       <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="177"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -183,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,9 +225,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -922,38 +937,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="טבלה1" displayName="טבלה1" ref="B7:AD69" headerRowCount="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30" tableBorderDxfId="29">
-  <autoFilter ref="B7:AD69"/>
-  <tableColumns count="29">
-    <tableColumn id="1" name="עמודה1" dataDxfId="28"/>
-    <tableColumn id="2" name="עמודה2" dataDxfId="27"/>
-    <tableColumn id="5" name="עמודה5" dataDxfId="26"/>
-    <tableColumn id="6" name="עמודה6" dataDxfId="25"/>
-    <tableColumn id="4" name="עמודה62" dataDxfId="24"/>
-    <tableColumn id="3" name="עמודה7" dataDxfId="23"/>
-    <tableColumn id="9" name="עמודה9" dataDxfId="22"/>
-    <tableColumn id="28" name="עמודה94" dataDxfId="21"/>
-    <tableColumn id="27" name="עמודה93" dataDxfId="20"/>
-    <tableColumn id="29" name="עמודה932" dataDxfId="19"/>
-    <tableColumn id="26" name="עמודה92" dataDxfId="18"/>
-    <tableColumn id="31" name="עמודה923" dataDxfId="17"/>
-    <tableColumn id="30" name="עמודה922" dataDxfId="16"/>
-    <tableColumn id="10" name="עמודה10" dataDxfId="15"/>
-    <tableColumn id="11" name="עמודה11" dataDxfId="14"/>
-    <tableColumn id="12" name="עמודה12" dataDxfId="13"/>
-    <tableColumn id="13" name="עמודה13" dataDxfId="12"/>
-    <tableColumn id="14" name="עמודה14" dataDxfId="11"/>
-    <tableColumn id="15" name="עמודה15" dataDxfId="10"/>
-    <tableColumn id="16" name="עמודה16" dataDxfId="9"/>
-    <tableColumn id="17" name="עמודה17" dataDxfId="8"/>
-    <tableColumn id="18" name="עמודה18" dataDxfId="7"/>
-    <tableColumn id="19" name="עמודה19" dataDxfId="6"/>
-    <tableColumn id="20" name="עמודה20" dataDxfId="5"/>
-    <tableColumn id="21" name="עמודה21" dataDxfId="4"/>
-    <tableColumn id="22" name="עמודה22" dataDxfId="3"/>
-    <tableColumn id="23" name="עמודה23" dataDxfId="2"/>
-    <tableColumn id="24" name="עמודה24" dataDxfId="1"/>
-    <tableColumn id="25" name="עמודה25" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="טבלה1" displayName="טבלה1" ref="B7:AG69" headerRowCount="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30" tableBorderDxfId="29">
+  <autoFilter ref="B7:AG69"/>
+  <tableColumns count="32">
+    <tableColumn id="1" name="עמודה1"/>
+    <tableColumn id="2" name="התחלה"/>
+    <tableColumn id="3" name="סיום"/>
+    <tableColumn id="4" name="סה&quot;כ שעות"/>
+    <tableColumn id="5" name="עמודה2"/>
+    <tableColumn id="6" name="עמודה5"/>
+    <tableColumn id="7" name="עמודה6"/>
+    <tableColumn id="8" name="עמודה62"/>
+    <tableColumn id="9" name="עמודה7"/>
+    <tableColumn id="10" name="עמודה9"/>
+    <tableColumn id="11" name="עמודה94"/>
+    <tableColumn id="12" name="עמודה93"/>
+    <tableColumn id="13" name="עמודה932"/>
+    <tableColumn id="14" name="עמודה92"/>
+    <tableColumn id="15" name="עמודה923"/>
+    <tableColumn id="16" name="עמודה922"/>
+    <tableColumn id="17" name="עמודה10"/>
+    <tableColumn id="18" name="עמודה11"/>
+    <tableColumn id="19" name="עמודה12"/>
+    <tableColumn id="20" name="עמודה13"/>
+    <tableColumn id="21" name="עמודה14"/>
+    <tableColumn id="22" name="עמודה15"/>
+    <tableColumn id="23" name="עמודה16"/>
+    <tableColumn id="24" name="עמודה17"/>
+    <tableColumn id="25" name="עמודה18"/>
+    <tableColumn id="26" name="עמודה19"/>
+    <tableColumn id="27" name="עמודה20"/>
+    <tableColumn id="28" name="עמודה21"/>
+    <tableColumn id="29" name="עמודה22"/>
+    <tableColumn id="30" name="עמודה23"/>
+    <tableColumn id="31" name="עמודה24"/>
+    <tableColumn id="32" name="עמודה25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1226,36 +1244,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:AE69"/>
+  <dimension ref="A1:AG72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="10.3984375" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="11.8984375" customWidth="1" min="3" max="3"/>
-    <col width="13.09765625" customWidth="1" min="4" max="4"/>
-    <col width="14.19921875" customWidth="1" min="5" max="7"/>
-    <col width="11.5" customWidth="1" min="8" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="7"/>
+    <col width="11.8984375" customWidth="1" min="6" max="6"/>
+    <col width="13.09765625" customWidth="1" min="7" max="7"/>
+    <col width="14.19921875" customWidth="1" min="8" max="10"/>
+    <col width="11.5" customWidth="1" min="11" max="11"/>
     <col width="14.8984375" bestFit="1" customWidth="1" min="12" max="12"/>
     <col width="14.3984375" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="11.5" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15.3984375" customWidth="1" min="16" max="16"/>
-    <col width="15.09765625" customWidth="1" min="17" max="17"/>
-    <col width="15.69921875" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="11.3984375" customWidth="1" min="20" max="20"/>
-    <col width="9.5" customWidth="1" min="21" max="25"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14.8984375" customWidth="1" min="15" max="15"/>
+    <col width="14.3984375" customWidth="1" min="16" max="16"/>
+    <col width="11.5" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15.3984375" customWidth="1" min="19" max="19"/>
+    <col width="15.09765625" customWidth="1" min="20" max="20"/>
+    <col width="15.69921875" customWidth="1" min="21" max="25"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="11.3984375" customWidth="1" min="23" max="23"/>
+    <col width="9.5" customWidth="1" min="24" max="24"/>
     <col width="11.09765625" customWidth="1" min="26" max="27"/>
     <col width="9.5" customWidth="1" min="28" max="30"/>
+    <col width="11.09765625" customWidth="1" min="29" max="29"/>
+    <col width="9.5" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4">
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="18" t="n"/>
-      <c r="F4" s="18" t="n"/>
-      <c r="G4" s="18" t="n"/>
-    </row>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="18" t="n"/>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
@@ -1269,140 +1299,155 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
+          <t>התחלה</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>סיום</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>סה"כ שעות</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
           <t>עמודה2</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>עמודה5</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>עמודה6</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>עמודה62</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>עמודה7</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>עמודה9</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>עמודה94</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>עמודה93</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="N7" s="9" t="inlineStr">
         <is>
           <t>עמודה932</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>עמודה92</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>עמודה923</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>עמודה922</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="R7" s="9" t="inlineStr">
         <is>
           <t>עמודה10</t>
         </is>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="S7" s="9" t="inlineStr">
         <is>
           <t>עמודה11</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="T7" s="9" t="inlineStr">
         <is>
           <t>עמודה12</t>
         </is>
       </c>
-      <c r="R7" s="9" t="inlineStr">
+      <c r="U7" s="9" t="inlineStr">
         <is>
           <t>עמודה13</t>
         </is>
       </c>
-      <c r="S7" s="9" t="inlineStr">
+      <c r="V7" s="9" t="inlineStr">
         <is>
           <t>עמודה14</t>
         </is>
       </c>
-      <c r="T7" s="9" t="inlineStr">
+      <c r="W7" s="9" t="inlineStr">
         <is>
           <t>עמודה15</t>
         </is>
       </c>
-      <c r="U7" s="9" t="inlineStr">
+      <c r="X7" s="9" t="inlineStr">
         <is>
           <t>עמודה16</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="Y7" s="2" t="inlineStr">
         <is>
           <t>עמודה17</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>עמודה18</t>
         </is>
       </c>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="AA7" s="2" t="inlineStr">
         <is>
           <t>עמודה19</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr">
+      <c r="AB7" s="2" t="inlineStr">
         <is>
           <t>עמודה20</t>
         </is>
       </c>
-      <c r="Z7" s="2" t="inlineStr">
+      <c r="AC7" s="2" t="inlineStr">
         <is>
           <t>עמודה21</t>
         </is>
       </c>
-      <c r="AA7" s="2" t="inlineStr">
+      <c r="AD7" s="2" t="inlineStr">
         <is>
           <t>עמודה22</t>
         </is>
       </c>
-      <c r="AB7" s="2" t="inlineStr">
+      <c r="AE7" s="2" t="inlineStr">
         <is>
           <t>עמודה23</t>
         </is>
       </c>
-      <c r="AC7" s="3" t="inlineStr">
+      <c r="AF7" s="3" t="inlineStr">
         <is>
           <t>עמודה24</t>
         </is>
       </c>
-      <c r="AD7" s="3" t="inlineStr">
+      <c r="AG7" s="3" t="inlineStr">
         <is>
           <t>עמודה25</t>
         </is>
@@ -1416,100 +1461,118 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
+          <t>התחלה</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>סיום</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>סה"כ שעות</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
           <t>ע הפקה ג</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>ע הפקה ג</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ע הפקה </t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ע הפקה </t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">נערת מים </t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="K8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">צלם 1 </t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>צלם 2</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">צלם 3 </t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ע צלם </t>
         </is>
       </c>
-      <c r="L8" s="9" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>ע צלם  2</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="P8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">מקליט </t>
         </is>
       </c>
-      <c r="N8" s="9" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>בום</t>
         </is>
       </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="R8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">תאורן </t>
         </is>
       </c>
-      <c r="P8" s="9" t="inlineStr">
+      <c r="S8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ע תאורן </t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="T8" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">גריפ </t>
         </is>
       </c>
-      <c r="R8" s="9" t="n"/>
-      <c r="S8" s="9" t="n"/>
-      <c r="T8" s="9" t="n"/>
       <c r="U8" s="9" t="n"/>
-      <c r="V8" s="2" t="n"/>
-      <c r="W8" s="2" t="n"/>
-      <c r="X8" s="2" t="n"/>
+      <c r="V8" s="9" t="n"/>
+      <c r="W8" s="9" t="n"/>
+      <c r="X8" s="9" t="n"/>
       <c r="Y8" s="2" t="n"/>
       <c r="Z8" s="2" t="n"/>
       <c r="AA8" s="2" t="n"/>
       <c r="AB8" s="2" t="n"/>
-      <c r="AC8" s="3" t="n"/>
-      <c r="AD8" s="3" t="n"/>
+      <c r="AC8" s="2" t="n"/>
+      <c r="AD8" s="2" t="n"/>
+      <c r="AE8" s="2" t="n"/>
+      <c r="AF8" s="3" t="n"/>
+      <c r="AG8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="27" t="n">
         <v>46296</v>
       </c>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="28">
+        <f>IF(OR(C9="",D9=""),"",MOD(D9-C9,1))</f>
+        <v/>
+      </c>
       <c r="F9" s="15" t="n"/>
       <c r="G9" s="15" t="n"/>
       <c r="H9" s="15" t="n"/>
@@ -1533,16 +1596,22 @@
       <c r="Z9" s="15" t="n"/>
       <c r="AA9" s="15" t="n"/>
       <c r="AB9" s="15" t="n"/>
-      <c r="AC9" s="3" t="n"/>
-      <c r="AD9" s="3" t="n"/>
+      <c r="AC9" s="15" t="n"/>
+      <c r="AD9" s="15" t="n"/>
+      <c r="AE9" s="15" t="n"/>
+      <c r="AF9" s="3" t="n"/>
+      <c r="AG9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="27" t="n">
         <v>46297</v>
       </c>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="28">
+        <f>IF(OR(C10="",D10=""),"",MOD(D10-C10,1))</f>
+        <v/>
+      </c>
       <c r="F10" s="15" t="n"/>
       <c r="G10" s="15" t="n"/>
       <c r="H10" s="15" t="n"/>
@@ -1566,16 +1635,22 @@
       <c r="Z10" s="15" t="n"/>
       <c r="AA10" s="15" t="n"/>
       <c r="AB10" s="15" t="n"/>
-      <c r="AC10" s="3" t="n"/>
-      <c r="AD10" s="3" t="n"/>
+      <c r="AC10" s="15" t="n"/>
+      <c r="AD10" s="15" t="n"/>
+      <c r="AE10" s="15" t="n"/>
+      <c r="AF10" s="3" t="n"/>
+      <c r="AG10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="27" t="n">
         <v>46298</v>
       </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="28">
+        <f>IF(OR(C11="",D11=""),"",MOD(D11-C11,1))</f>
+        <v/>
+      </c>
       <c r="F11" s="15" t="n"/>
       <c r="G11" s="15" t="n"/>
       <c r="H11" s="15" t="n"/>
@@ -1599,16 +1674,22 @@
       <c r="Z11" s="15" t="n"/>
       <c r="AA11" s="15" t="n"/>
       <c r="AB11" s="15" t="n"/>
-      <c r="AC11" s="3" t="n"/>
-      <c r="AD11" s="3" t="n"/>
+      <c r="AC11" s="15" t="n"/>
+      <c r="AD11" s="15" t="n"/>
+      <c r="AE11" s="15" t="n"/>
+      <c r="AF11" s="3" t="n"/>
+      <c r="AG11" s="3" t="n"/>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="27" t="n">
         <v>46299</v>
       </c>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="28">
+        <f>IF(OR(C12="",D12=""),"",MOD(D12-C12,1))</f>
+        <v/>
+      </c>
       <c r="F12" s="15" t="n"/>
       <c r="G12" s="15" t="n"/>
       <c r="H12" s="15" t="n"/>
@@ -1632,16 +1713,22 @@
       <c r="Z12" s="15" t="n"/>
       <c r="AA12" s="15" t="n"/>
       <c r="AB12" s="15" t="n"/>
-      <c r="AC12" s="3" t="n"/>
-      <c r="AD12" s="3" t="n"/>
+      <c r="AC12" s="15" t="n"/>
+      <c r="AD12" s="15" t="n"/>
+      <c r="AE12" s="15" t="n"/>
+      <c r="AF12" s="3" t="n"/>
+      <c r="AG12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="27" t="n">
         <v>46300</v>
       </c>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="28">
+        <f>IF(OR(C13="",D13=""),"",MOD(D13-C13,1))</f>
+        <v/>
+      </c>
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
       <c r="H13" s="15" t="n"/>
@@ -1665,16 +1752,22 @@
       <c r="Z13" s="15" t="n"/>
       <c r="AA13" s="15" t="n"/>
       <c r="AB13" s="15" t="n"/>
-      <c r="AC13" s="3" t="n"/>
-      <c r="AD13" s="3" t="n"/>
+      <c r="AC13" s="15" t="n"/>
+      <c r="AD13" s="15" t="n"/>
+      <c r="AE13" s="15" t="n"/>
+      <c r="AF13" s="3" t="n"/>
+      <c r="AG13" s="3" t="n"/>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="27" t="n">
         <v>46301</v>
       </c>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
-      <c r="E14" s="15" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="28">
+        <f>IF(OR(C14="",D14=""),"",MOD(D14-C14,1))</f>
+        <v/>
+      </c>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
       <c r="H14" s="15" t="n"/>
@@ -1698,16 +1791,22 @@
       <c r="Z14" s="15" t="n"/>
       <c r="AA14" s="15" t="n"/>
       <c r="AB14" s="15" t="n"/>
-      <c r="AC14" s="3" t="n"/>
-      <c r="AD14" s="3" t="n"/>
+      <c r="AC14" s="15" t="n"/>
+      <c r="AD14" s="15" t="n"/>
+      <c r="AE14" s="15" t="n"/>
+      <c r="AF14" s="3" t="n"/>
+      <c r="AG14" s="3" t="n"/>
     </row>
     <row r="15" ht="18.75" customHeight="1">
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="27" t="n">
         <v>46302</v>
       </c>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="28">
+        <f>IF(OR(C15="",D15=""),"",MOD(D15-C15,1))</f>
+        <v/>
+      </c>
       <c r="F15" s="15" t="n"/>
       <c r="G15" s="15" t="n"/>
       <c r="H15" s="15" t="n"/>
@@ -1731,16 +1830,22 @@
       <c r="Z15" s="15" t="n"/>
       <c r="AA15" s="15" t="n"/>
       <c r="AB15" s="15" t="n"/>
-      <c r="AC15" s="3" t="n"/>
-      <c r="AD15" s="3" t="n"/>
+      <c r="AC15" s="15" t="n"/>
+      <c r="AD15" s="15" t="n"/>
+      <c r="AE15" s="15" t="n"/>
+      <c r="AF15" s="3" t="n"/>
+      <c r="AG15" s="3" t="n"/>
     </row>
     <row r="16" ht="17.25" customHeight="1">
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="27" t="n">
         <v>46303</v>
       </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="28">
+        <f>IF(OR(C16="",D16=""),"",MOD(D16-C16,1))</f>
+        <v/>
+      </c>
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
       <c r="H16" s="15" t="n"/>
@@ -1764,16 +1869,22 @@
       <c r="Z16" s="15" t="n"/>
       <c r="AA16" s="15" t="n"/>
       <c r="AB16" s="15" t="n"/>
-      <c r="AC16" s="3" t="n"/>
-      <c r="AD16" s="3" t="n"/>
+      <c r="AC16" s="15" t="n"/>
+      <c r="AD16" s="15" t="n"/>
+      <c r="AE16" s="15" t="n"/>
+      <c r="AF16" s="3" t="n"/>
+      <c r="AG16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="27" t="n">
         <v>46304</v>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="28">
+        <f>IF(OR(C17="",D17=""),"",MOD(D17-C17,1))</f>
+        <v/>
+      </c>
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
       <c r="H17" s="15" t="n"/>
@@ -1797,16 +1908,22 @@
       <c r="Z17" s="15" t="n"/>
       <c r="AA17" s="15" t="n"/>
       <c r="AB17" s="15" t="n"/>
-      <c r="AC17" s="3" t="n"/>
-      <c r="AD17" s="3" t="n"/>
+      <c r="AC17" s="15" t="n"/>
+      <c r="AD17" s="15" t="n"/>
+      <c r="AE17" s="15" t="n"/>
+      <c r="AF17" s="3" t="n"/>
+      <c r="AG17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="24" t="n">
+      <c r="B18" s="27" t="n">
         <v>46305</v>
       </c>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="28">
+        <f>IF(OR(C18="",D18=""),"",MOD(D18-C18,1))</f>
+        <v/>
+      </c>
       <c r="F18" s="15" t="n"/>
       <c r="G18" s="15" t="n"/>
       <c r="H18" s="15" t="n"/>
@@ -1830,16 +1947,22 @@
       <c r="Z18" s="15" t="n"/>
       <c r="AA18" s="15" t="n"/>
       <c r="AB18" s="15" t="n"/>
-      <c r="AC18" s="3" t="n"/>
-      <c r="AD18" s="3" t="n"/>
+      <c r="AC18" s="15" t="n"/>
+      <c r="AD18" s="15" t="n"/>
+      <c r="AE18" s="15" t="n"/>
+      <c r="AF18" s="3" t="n"/>
+      <c r="AG18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="27" t="n">
         <v>46306</v>
       </c>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="28">
+        <f>IF(OR(C19="",D19=""),"",MOD(D19-C19,1))</f>
+        <v/>
+      </c>
       <c r="F19" s="15" t="n"/>
       <c r="G19" s="15" t="n"/>
       <c r="H19" s="15" t="n"/>
@@ -1863,16 +1986,26 @@
       <c r="Z19" s="15" t="n"/>
       <c r="AA19" s="15" t="n"/>
       <c r="AB19" s="15" t="n"/>
-      <c r="AC19" s="3" t="n"/>
-      <c r="AD19" s="3" t="n"/>
+      <c r="AC19" s="15" t="n"/>
+      <c r="AD19" s="15" t="n"/>
+      <c r="AE19" s="15" t="n"/>
+      <c r="AF19" s="3" t="n"/>
+      <c r="AG19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="24" t="n">
+      <c r="B20" s="27" t="n">
         <v>46307</v>
       </c>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
+      <c r="C20" s="21" t="n">
+        <v>0.2916666666666667</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="E20" s="28">
+        <f>IF(OR(C20="",D20=""),"",MOD(D20-C20,1))</f>
+        <v/>
+      </c>
       <c r="F20" s="15" t="n"/>
       <c r="G20" s="15" t="n"/>
       <c r="H20" s="15" t="n"/>
@@ -1896,16 +2029,26 @@
       <c r="Z20" s="15" t="n"/>
       <c r="AA20" s="15" t="n"/>
       <c r="AB20" s="15" t="n"/>
-      <c r="AC20" s="3" t="n"/>
-      <c r="AD20" s="3" t="n"/>
+      <c r="AC20" s="15" t="n"/>
+      <c r="AD20" s="15" t="n"/>
+      <c r="AE20" s="15" t="n"/>
+      <c r="AF20" s="3" t="n"/>
+      <c r="AG20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="24" t="n">
+      <c r="B21" s="27" t="n">
         <v>46308</v>
       </c>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="15" t="n"/>
+      <c r="C21" s="21" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E21" s="28">
+        <f>IF(OR(C21="",D21=""),"",MOD(D21-C21,1))</f>
+        <v/>
+      </c>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="15" t="n"/>
@@ -1929,16 +2072,26 @@
       <c r="Z21" s="15" t="n"/>
       <c r="AA21" s="15" t="n"/>
       <c r="AB21" s="15" t="n"/>
-      <c r="AC21" s="3" t="n"/>
-      <c r="AD21" s="3" t="n"/>
+      <c r="AC21" s="15" t="n"/>
+      <c r="AD21" s="15" t="n"/>
+      <c r="AE21" s="15" t="n"/>
+      <c r="AF21" s="3" t="n"/>
+      <c r="AG21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="24" t="n">
+      <c r="B22" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
+      <c r="C22" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>0.7638888888888888</v>
+      </c>
+      <c r="E22" s="28">
+        <f>IF(OR(C22="",D22=""),"",MOD(D22-C22,1))</f>
+        <v/>
+      </c>
       <c r="F22" s="15" t="n"/>
       <c r="G22" s="15" t="n"/>
       <c r="H22" s="15" t="n"/>
@@ -1962,16 +2115,26 @@
       <c r="Z22" s="15" t="n"/>
       <c r="AA22" s="15" t="n"/>
       <c r="AB22" s="15" t="n"/>
-      <c r="AC22" s="3" t="n"/>
-      <c r="AD22" s="3" t="n"/>
+      <c r="AC22" s="15" t="n"/>
+      <c r="AD22" s="15" t="n"/>
+      <c r="AE22" s="15" t="n"/>
+      <c r="AF22" s="3" t="n"/>
+      <c r="AG22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="24" t="n">
+      <c r="B23" s="27" t="n">
         <v>46310</v>
       </c>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
+      <c r="C23" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>0.8194444444444444</v>
+      </c>
+      <c r="E23" s="28">
+        <f>IF(OR(C23="",D23=""),"",MOD(D23-C23,1))</f>
+        <v/>
+      </c>
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
       <c r="H23" s="15" t="n"/>
@@ -1995,16 +2158,22 @@
       <c r="Z23" s="15" t="n"/>
       <c r="AA23" s="15" t="n"/>
       <c r="AB23" s="15" t="n"/>
-      <c r="AC23" s="3" t="n"/>
-      <c r="AD23" s="3" t="n"/>
+      <c r="AC23" s="15" t="n"/>
+      <c r="AD23" s="15" t="n"/>
+      <c r="AE23" s="15" t="n"/>
+      <c r="AF23" s="3" t="n"/>
+      <c r="AG23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="24" t="n">
+      <c r="B24" s="27" t="n">
         <v>46311</v>
       </c>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="28">
+        <f>IF(OR(C24="",D24=""),"",MOD(D24-C24,1))</f>
+        <v/>
+      </c>
       <c r="F24" s="15" t="n"/>
       <c r="G24" s="15" t="n"/>
       <c r="H24" s="15" t="n"/>
@@ -2028,16 +2197,22 @@
       <c r="Z24" s="15" t="n"/>
       <c r="AA24" s="15" t="n"/>
       <c r="AB24" s="15" t="n"/>
-      <c r="AC24" s="3" t="n"/>
-      <c r="AD24" s="3" t="n"/>
+      <c r="AC24" s="15" t="n"/>
+      <c r="AD24" s="15" t="n"/>
+      <c r="AE24" s="15" t="n"/>
+      <c r="AF24" s="3" t="n"/>
+      <c r="AG24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="24" t="n">
+      <c r="B25" s="27" t="n">
         <v>46312</v>
       </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="28">
+        <f>IF(OR(C25="",D25=""),"",MOD(D25-C25,1))</f>
+        <v/>
+      </c>
       <c r="F25" s="15" t="n"/>
       <c r="G25" s="15" t="n"/>
       <c r="H25" s="15" t="n"/>
@@ -2061,16 +2236,26 @@
       <c r="Z25" s="15" t="n"/>
       <c r="AA25" s="15" t="n"/>
       <c r="AB25" s="15" t="n"/>
-      <c r="AC25" s="3" t="n"/>
-      <c r="AD25" s="3" t="n"/>
+      <c r="AC25" s="15" t="n"/>
+      <c r="AD25" s="15" t="n"/>
+      <c r="AE25" s="15" t="n"/>
+      <c r="AF25" s="3" t="n"/>
+      <c r="AG25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="24" t="n">
+      <c r="B26" s="27" t="n">
         <v>46313</v>
       </c>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
+      <c r="C26" s="21" t="n">
+        <v>0.1458333333333333</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E26" s="28">
+        <f>IF(OR(C26="",D26=""),"",MOD(D26-C26,1))</f>
+        <v/>
+      </c>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
       <c r="H26" s="15" t="n"/>
@@ -2094,16 +2279,26 @@
       <c r="Z26" s="15" t="n"/>
       <c r="AA26" s="15" t="n"/>
       <c r="AB26" s="15" t="n"/>
-      <c r="AC26" s="3" t="n"/>
-      <c r="AD26" s="3" t="n"/>
+      <c r="AC26" s="15" t="n"/>
+      <c r="AD26" s="15" t="n"/>
+      <c r="AE26" s="15" t="n"/>
+      <c r="AF26" s="3" t="n"/>
+      <c r="AG26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="24" t="n">
+      <c r="B27" s="27" t="n">
         <v>46314</v>
       </c>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
+      <c r="C27" s="21" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>0.6805555555555556</v>
+      </c>
+      <c r="E27" s="28">
+        <f>IF(OR(C27="",D27=""),"",MOD(D27-C27,1))</f>
+        <v/>
+      </c>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="15" t="n"/>
@@ -2127,16 +2322,26 @@
       <c r="Z27" s="15" t="n"/>
       <c r="AA27" s="15" t="n"/>
       <c r="AB27" s="15" t="n"/>
-      <c r="AC27" s="3" t="n"/>
-      <c r="AD27" s="3" t="n"/>
+      <c r="AC27" s="15" t="n"/>
+      <c r="AD27" s="15" t="n"/>
+      <c r="AE27" s="15" t="n"/>
+      <c r="AF27" s="3" t="n"/>
+      <c r="AG27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="24" t="n">
+      <c r="B28" s="27" t="n">
         <v>46315</v>
       </c>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
+      <c r="C28" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E28" s="28">
+        <f>IF(OR(C28="",D28=""),"",MOD(D28-C28,1))</f>
+        <v/>
+      </c>
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
       <c r="H28" s="15" t="n"/>
@@ -2160,16 +2365,26 @@
       <c r="Z28" s="15" t="n"/>
       <c r="AA28" s="15" t="n"/>
       <c r="AB28" s="15" t="n"/>
-      <c r="AC28" s="3" t="n"/>
-      <c r="AD28" s="3" t="n"/>
+      <c r="AC28" s="15" t="n"/>
+      <c r="AD28" s="15" t="n"/>
+      <c r="AE28" s="15" t="n"/>
+      <c r="AF28" s="3" t="n"/>
+      <c r="AG28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="24" t="n">
+      <c r="B29" s="27" t="n">
         <v>46316</v>
       </c>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
+      <c r="C29" s="21" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="D29" s="21" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="E29" s="28">
+        <f>IF(OR(C29="",D29=""),"",MOD(D29-C29,1))</f>
+        <v/>
+      </c>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
       <c r="H29" s="15" t="n"/>
@@ -2193,16 +2408,26 @@
       <c r="Z29" s="15" t="n"/>
       <c r="AA29" s="15" t="n"/>
       <c r="AB29" s="15" t="n"/>
-      <c r="AC29" s="3" t="n"/>
-      <c r="AD29" s="3" t="n"/>
+      <c r="AC29" s="15" t="n"/>
+      <c r="AD29" s="15" t="n"/>
+      <c r="AE29" s="15" t="n"/>
+      <c r="AF29" s="3" t="n"/>
+      <c r="AG29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="24" t="n">
+      <c r="B30" s="27" t="n">
         <v>46317</v>
       </c>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
+      <c r="C30" s="21" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="D30" s="21" t="n">
+        <v>0.8194444444444444</v>
+      </c>
+      <c r="E30" s="28">
+        <f>IF(OR(C30="",D30=""),"",MOD(D30-C30,1))</f>
+        <v/>
+      </c>
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
       <c r="H30" s="15" t="n"/>
@@ -2226,16 +2451,22 @@
       <c r="Z30" s="15" t="n"/>
       <c r="AA30" s="15" t="n"/>
       <c r="AB30" s="15" t="n"/>
-      <c r="AC30" s="3" t="n"/>
-      <c r="AD30" s="3" t="n"/>
+      <c r="AC30" s="15" t="n"/>
+      <c r="AD30" s="15" t="n"/>
+      <c r="AE30" s="15" t="n"/>
+      <c r="AF30" s="3" t="n"/>
+      <c r="AG30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="24" t="n">
+      <c r="B31" s="27" t="n">
         <v>46318</v>
       </c>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="28">
+        <f>IF(OR(C31="",D31=""),"",MOD(D31-C31,1))</f>
+        <v/>
+      </c>
       <c r="F31" s="15" t="n"/>
       <c r="G31" s="15" t="n"/>
       <c r="H31" s="15" t="n"/>
@@ -2259,16 +2490,22 @@
       <c r="Z31" s="15" t="n"/>
       <c r="AA31" s="15" t="n"/>
       <c r="AB31" s="15" t="n"/>
-      <c r="AC31" s="3" t="n"/>
-      <c r="AD31" s="3" t="n"/>
+      <c r="AC31" s="15" t="n"/>
+      <c r="AD31" s="15" t="n"/>
+      <c r="AE31" s="15" t="n"/>
+      <c r="AF31" s="3" t="n"/>
+      <c r="AG31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="24" t="n">
+      <c r="B32" s="27" t="n">
         <v>46319</v>
       </c>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
+      <c r="C32" s="21" t="n"/>
+      <c r="D32" s="21" t="n"/>
+      <c r="E32" s="28">
+        <f>IF(OR(C32="",D32=""),"",MOD(D32-C32,1))</f>
+        <v/>
+      </c>
       <c r="F32" s="15" t="n"/>
       <c r="G32" s="15" t="n"/>
       <c r="H32" s="15" t="n"/>
@@ -2292,16 +2529,26 @@
       <c r="Z32" s="15" t="n"/>
       <c r="AA32" s="15" t="n"/>
       <c r="AB32" s="15" t="n"/>
-      <c r="AC32" s="3" t="n"/>
-      <c r="AD32" s="3" t="n"/>
+      <c r="AC32" s="15" t="n"/>
+      <c r="AD32" s="15" t="n"/>
+      <c r="AE32" s="15" t="n"/>
+      <c r="AF32" s="3" t="n"/>
+      <c r="AG32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="24" t="n">
+      <c r="B33" s="27" t="n">
         <v>46320</v>
       </c>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
+      <c r="C33" s="21" t="n">
+        <v>0.1805555555555556</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="E33" s="28">
+        <f>IF(OR(C33="",D33=""),"",MOD(D33-C33,1))</f>
+        <v/>
+      </c>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n"/>
       <c r="H33" s="15" t="n"/>
@@ -2325,16 +2572,26 @@
       <c r="Z33" s="15" t="n"/>
       <c r="AA33" s="15" t="n"/>
       <c r="AB33" s="15" t="n"/>
-      <c r="AC33" s="3" t="n"/>
-      <c r="AD33" s="3" t="n"/>
+      <c r="AC33" s="15" t="n"/>
+      <c r="AD33" s="15" t="n"/>
+      <c r="AE33" s="15" t="n"/>
+      <c r="AF33" s="3" t="n"/>
+      <c r="AG33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="24" t="n">
+      <c r="B34" s="27" t="n">
         <v>46321</v>
       </c>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
+      <c r="C34" s="21" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="E34" s="28">
+        <f>IF(OR(C34="",D34=""),"",MOD(D34-C34,1))</f>
+        <v/>
+      </c>
       <c r="F34" s="15" t="n"/>
       <c r="G34" s="15" t="n"/>
       <c r="H34" s="15" t="n"/>
@@ -2358,16 +2615,22 @@
       <c r="Z34" s="15" t="n"/>
       <c r="AA34" s="15" t="n"/>
       <c r="AB34" s="15" t="n"/>
-      <c r="AC34" s="3" t="n"/>
-      <c r="AD34" s="3" t="n"/>
+      <c r="AC34" s="15" t="n"/>
+      <c r="AD34" s="15" t="n"/>
+      <c r="AE34" s="15" t="n"/>
+      <c r="AF34" s="3" t="n"/>
+      <c r="AG34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="24" t="n">
+      <c r="B35" s="27" t="n">
         <v>46322</v>
       </c>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="21" t="n"/>
+      <c r="E35" s="28">
+        <f>IF(OR(C35="",D35=""),"",MOD(D35-C35,1))</f>
+        <v/>
+      </c>
       <c r="F35" s="15" t="n"/>
       <c r="G35" s="15" t="n"/>
       <c r="H35" s="15" t="n"/>
@@ -2391,16 +2654,22 @@
       <c r="Z35" s="15" t="n"/>
       <c r="AA35" s="15" t="n"/>
       <c r="AB35" s="15" t="n"/>
-      <c r="AC35" s="3" t="n"/>
-      <c r="AD35" s="3" t="n"/>
+      <c r="AC35" s="15" t="n"/>
+      <c r="AD35" s="15" t="n"/>
+      <c r="AE35" s="15" t="n"/>
+      <c r="AF35" s="3" t="n"/>
+      <c r="AG35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="24" t="n">
+      <c r="B36" s="27" t="n">
         <v>46323</v>
       </c>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
+      <c r="C36" s="21" t="n"/>
+      <c r="D36" s="21" t="n"/>
+      <c r="E36" s="28">
+        <f>IF(OR(C36="",D36=""),"",MOD(D36-C36,1))</f>
+        <v/>
+      </c>
       <c r="F36" s="15" t="n"/>
       <c r="G36" s="15" t="n"/>
       <c r="H36" s="15" t="n"/>
@@ -2424,16 +2693,22 @@
       <c r="Z36" s="15" t="n"/>
       <c r="AA36" s="15" t="n"/>
       <c r="AB36" s="15" t="n"/>
-      <c r="AC36" s="3" t="n"/>
-      <c r="AD36" s="3" t="n"/>
+      <c r="AC36" s="15" t="n"/>
+      <c r="AD36" s="15" t="n"/>
+      <c r="AE36" s="15" t="n"/>
+      <c r="AF36" s="3" t="n"/>
+      <c r="AG36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="24" t="n">
+      <c r="B37" s="27" t="n">
         <v>46324</v>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
+      <c r="C37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+      <c r="E37" s="28">
+        <f>IF(OR(C37="",D37=""),"",MOD(D37-C37,1))</f>
+        <v/>
+      </c>
       <c r="F37" s="15" t="n"/>
       <c r="G37" s="15" t="n"/>
       <c r="H37" s="15" t="n"/>
@@ -2457,16 +2732,22 @@
       <c r="Z37" s="15" t="n"/>
       <c r="AA37" s="15" t="n"/>
       <c r="AB37" s="15" t="n"/>
-      <c r="AC37" s="3" t="n"/>
-      <c r="AD37" s="3" t="n"/>
+      <c r="AC37" s="15" t="n"/>
+      <c r="AD37" s="15" t="n"/>
+      <c r="AE37" s="15" t="n"/>
+      <c r="AF37" s="3" t="n"/>
+      <c r="AG37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="24" t="n">
+      <c r="B38" s="27" t="n">
         <v>46325</v>
       </c>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
+      <c r="C38" s="21" t="n"/>
+      <c r="D38" s="21" t="n"/>
+      <c r="E38" s="28">
+        <f>IF(OR(C38="",D38=""),"",MOD(D38-C38,1))</f>
+        <v/>
+      </c>
       <c r="F38" s="15" t="n"/>
       <c r="G38" s="15" t="n"/>
       <c r="H38" s="15" t="n"/>
@@ -2490,16 +2771,22 @@
       <c r="Z38" s="15" t="n"/>
       <c r="AA38" s="15" t="n"/>
       <c r="AB38" s="15" t="n"/>
-      <c r="AC38" s="3" t="n"/>
-      <c r="AD38" s="3" t="n"/>
+      <c r="AC38" s="15" t="n"/>
+      <c r="AD38" s="15" t="n"/>
+      <c r="AE38" s="15" t="n"/>
+      <c r="AF38" s="3" t="n"/>
+      <c r="AG38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="24" t="n">
+      <c r="B39" s="27" t="n">
         <v>46326</v>
       </c>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
+      <c r="C39" s="21" t="n"/>
+      <c r="D39" s="21" t="n"/>
+      <c r="E39" s="28">
+        <f>IF(OR(C39="",D39=""),"",MOD(D39-C39,1))</f>
+        <v/>
+      </c>
       <c r="F39" s="15" t="n"/>
       <c r="G39" s="15" t="n"/>
       <c r="H39" s="15" t="n"/>
@@ -2523,16 +2810,22 @@
       <c r="Z39" s="15" t="n"/>
       <c r="AA39" s="15" t="n"/>
       <c r="AB39" s="15" t="n"/>
-      <c r="AC39" s="3" t="n"/>
-      <c r="AD39" s="3" t="n"/>
+      <c r="AC39" s="15" t="n"/>
+      <c r="AD39" s="15" t="n"/>
+      <c r="AE39" s="15" t="n"/>
+      <c r="AF39" s="3" t="n"/>
+      <c r="AG39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="24" t="n">
+      <c r="B40" s="27" t="n">
         <v>46327</v>
       </c>
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="15" t="n"/>
-      <c r="E40" s="15" t="n"/>
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="28">
+        <f>IF(OR(C40="",D40=""),"",MOD(D40-C40,1))</f>
+        <v/>
+      </c>
       <c r="F40" s="15" t="n"/>
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="15" t="n"/>
@@ -2556,16 +2849,22 @@
       <c r="Z40" s="15" t="n"/>
       <c r="AA40" s="15" t="n"/>
       <c r="AB40" s="15" t="n"/>
-      <c r="AC40" s="3" t="n"/>
-      <c r="AD40" s="3" t="n"/>
+      <c r="AC40" s="15" t="n"/>
+      <c r="AD40" s="15" t="n"/>
+      <c r="AE40" s="15" t="n"/>
+      <c r="AF40" s="3" t="n"/>
+      <c r="AG40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="24" t="n">
+      <c r="B41" s="27" t="n">
         <v>46328</v>
       </c>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
+      <c r="C41" s="21" t="n"/>
+      <c r="D41" s="21" t="n"/>
+      <c r="E41" s="28">
+        <f>IF(OR(C41="",D41=""),"",MOD(D41-C41,1))</f>
+        <v/>
+      </c>
       <c r="F41" s="15" t="n"/>
       <c r="G41" s="15" t="n"/>
       <c r="H41" s="15" t="n"/>
@@ -2589,16 +2888,22 @@
       <c r="Z41" s="15" t="n"/>
       <c r="AA41" s="15" t="n"/>
       <c r="AB41" s="15" t="n"/>
-      <c r="AC41" s="3" t="n"/>
-      <c r="AD41" s="3" t="n"/>
+      <c r="AC41" s="15" t="n"/>
+      <c r="AD41" s="15" t="n"/>
+      <c r="AE41" s="15" t="n"/>
+      <c r="AF41" s="3" t="n"/>
+      <c r="AG41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="24" t="n">
+      <c r="B42" s="27" t="n">
         <v>46329</v>
       </c>
-      <c r="C42" s="15" t="n"/>
-      <c r="D42" s="15" t="n"/>
-      <c r="E42" s="15" t="n"/>
+      <c r="C42" s="21" t="n"/>
+      <c r="D42" s="21" t="n"/>
+      <c r="E42" s="28">
+        <f>IF(OR(C42="",D42=""),"",MOD(D42-C42,1))</f>
+        <v/>
+      </c>
       <c r="F42" s="15" t="n"/>
       <c r="G42" s="15" t="n"/>
       <c r="H42" s="15" t="n"/>
@@ -2622,16 +2927,22 @@
       <c r="Z42" s="15" t="n"/>
       <c r="AA42" s="15" t="n"/>
       <c r="AB42" s="15" t="n"/>
-      <c r="AC42" s="3" t="n"/>
-      <c r="AD42" s="3" t="n"/>
+      <c r="AC42" s="15" t="n"/>
+      <c r="AD42" s="15" t="n"/>
+      <c r="AE42" s="15" t="n"/>
+      <c r="AF42" s="3" t="n"/>
+      <c r="AG42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="24" t="n">
+      <c r="B43" s="27" t="n">
         <v>46330</v>
       </c>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="15" t="n"/>
-      <c r="E43" s="15" t="n"/>
+      <c r="C43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="28">
+        <f>IF(OR(C43="",D43=""),"",MOD(D43-C43,1))</f>
+        <v/>
+      </c>
       <c r="F43" s="15" t="n"/>
       <c r="G43" s="15" t="n"/>
       <c r="H43" s="15" t="n"/>
@@ -2655,16 +2966,22 @@
       <c r="Z43" s="15" t="n"/>
       <c r="AA43" s="15" t="n"/>
       <c r="AB43" s="15" t="n"/>
-      <c r="AC43" s="3" t="n"/>
-      <c r="AD43" s="3" t="n"/>
+      <c r="AC43" s="15" t="n"/>
+      <c r="AD43" s="15" t="n"/>
+      <c r="AE43" s="15" t="n"/>
+      <c r="AF43" s="3" t="n"/>
+      <c r="AG43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="24" t="n">
+      <c r="B44" s="27" t="n">
         <v>46331</v>
       </c>
-      <c r="C44" s="15" t="n"/>
-      <c r="D44" s="15" t="n"/>
-      <c r="E44" s="15" t="n"/>
+      <c r="C44" s="21" t="n"/>
+      <c r="D44" s="21" t="n"/>
+      <c r="E44" s="28">
+        <f>IF(OR(C44="",D44=""),"",MOD(D44-C44,1))</f>
+        <v/>
+      </c>
       <c r="F44" s="15" t="n"/>
       <c r="G44" s="15" t="n"/>
       <c r="H44" s="15" t="n"/>
@@ -2688,16 +3005,22 @@
       <c r="Z44" s="15" t="n"/>
       <c r="AA44" s="15" t="n"/>
       <c r="AB44" s="15" t="n"/>
-      <c r="AC44" s="3" t="n"/>
-      <c r="AD44" s="3" t="n"/>
+      <c r="AC44" s="15" t="n"/>
+      <c r="AD44" s="15" t="n"/>
+      <c r="AE44" s="15" t="n"/>
+      <c r="AF44" s="3" t="n"/>
+      <c r="AG44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="24" t="n">
+      <c r="B45" s="27" t="n">
         <v>46332</v>
       </c>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
+      <c r="C45" s="21" t="n"/>
+      <c r="D45" s="21" t="n"/>
+      <c r="E45" s="28">
+        <f>IF(OR(C45="",D45=""),"",MOD(D45-C45,1))</f>
+        <v/>
+      </c>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n"/>
       <c r="H45" s="15" t="n"/>
@@ -2721,16 +3044,22 @@
       <c r="Z45" s="15" t="n"/>
       <c r="AA45" s="15" t="n"/>
       <c r="AB45" s="15" t="n"/>
-      <c r="AC45" s="3" t="n"/>
-      <c r="AD45" s="3" t="n"/>
+      <c r="AC45" s="15" t="n"/>
+      <c r="AD45" s="15" t="n"/>
+      <c r="AE45" s="15" t="n"/>
+      <c r="AF45" s="3" t="n"/>
+      <c r="AG45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="24" t="n">
+      <c r="B46" s="27" t="n">
         <v>46333</v>
       </c>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
+      <c r="C46" s="21" t="n"/>
+      <c r="D46" s="21" t="n"/>
+      <c r="E46" s="28">
+        <f>IF(OR(C46="",D46=""),"",MOD(D46-C46,1))</f>
+        <v/>
+      </c>
       <c r="F46" s="15" t="n"/>
       <c r="G46" s="15" t="n"/>
       <c r="H46" s="15" t="n"/>
@@ -2754,16 +3083,22 @@
       <c r="Z46" s="15" t="n"/>
       <c r="AA46" s="15" t="n"/>
       <c r="AB46" s="15" t="n"/>
-      <c r="AC46" s="3" t="n"/>
-      <c r="AD46" s="3" t="n"/>
+      <c r="AC46" s="15" t="n"/>
+      <c r="AD46" s="15" t="n"/>
+      <c r="AE46" s="15" t="n"/>
+      <c r="AF46" s="3" t="n"/>
+      <c r="AG46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="24" t="n">
+      <c r="B47" s="27" t="n">
         <v>46334</v>
       </c>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
+      <c r="C47" s="21" t="n"/>
+      <c r="D47" s="21" t="n"/>
+      <c r="E47" s="28">
+        <f>IF(OR(C47="",D47=""),"",MOD(D47-C47,1))</f>
+        <v/>
+      </c>
       <c r="F47" s="15" t="n"/>
       <c r="G47" s="15" t="n"/>
       <c r="H47" s="15" t="n"/>
@@ -2787,16 +3122,22 @@
       <c r="Z47" s="15" t="n"/>
       <c r="AA47" s="15" t="n"/>
       <c r="AB47" s="15" t="n"/>
-      <c r="AC47" s="3" t="n"/>
-      <c r="AD47" s="3" t="n"/>
+      <c r="AC47" s="15" t="n"/>
+      <c r="AD47" s="15" t="n"/>
+      <c r="AE47" s="15" t="n"/>
+      <c r="AF47" s="3" t="n"/>
+      <c r="AG47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="24" t="n">
+      <c r="B48" s="27" t="n">
         <v>46335</v>
       </c>
-      <c r="C48" s="15" t="n"/>
-      <c r="D48" s="15" t="n"/>
-      <c r="E48" s="15" t="n"/>
+      <c r="C48" s="21" t="n"/>
+      <c r="D48" s="21" t="n"/>
+      <c r="E48" s="28">
+        <f>IF(OR(C48="",D48=""),"",MOD(D48-C48,1))</f>
+        <v/>
+      </c>
       <c r="F48" s="15" t="n"/>
       <c r="G48" s="15" t="n"/>
       <c r="H48" s="15" t="n"/>
@@ -2820,16 +3161,22 @@
       <c r="Z48" s="15" t="n"/>
       <c r="AA48" s="15" t="n"/>
       <c r="AB48" s="15" t="n"/>
-      <c r="AC48" s="3" t="n"/>
-      <c r="AD48" s="3" t="n"/>
+      <c r="AC48" s="15" t="n"/>
+      <c r="AD48" s="15" t="n"/>
+      <c r="AE48" s="15" t="n"/>
+      <c r="AF48" s="3" t="n"/>
+      <c r="AG48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="24" t="n">
+      <c r="B49" s="27" t="n">
         <v>46336</v>
       </c>
-      <c r="C49" s="15" t="n"/>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="15" t="n"/>
+      <c r="C49" s="21" t="n"/>
+      <c r="D49" s="21" t="n"/>
+      <c r="E49" s="28">
+        <f>IF(OR(C49="",D49=""),"",MOD(D49-C49,1))</f>
+        <v/>
+      </c>
       <c r="F49" s="15" t="n"/>
       <c r="G49" s="15" t="n"/>
       <c r="H49" s="15" t="n"/>
@@ -2853,16 +3200,22 @@
       <c r="Z49" s="15" t="n"/>
       <c r="AA49" s="15" t="n"/>
       <c r="AB49" s="15" t="n"/>
-      <c r="AC49" s="3" t="n"/>
-      <c r="AD49" s="3" t="n"/>
+      <c r="AC49" s="15" t="n"/>
+      <c r="AD49" s="15" t="n"/>
+      <c r="AE49" s="15" t="n"/>
+      <c r="AF49" s="3" t="n"/>
+      <c r="AG49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="24" t="n">
+      <c r="B50" s="27" t="n">
         <v>46337</v>
       </c>
-      <c r="C50" s="15" t="n"/>
-      <c r="D50" s="15" t="n"/>
-      <c r="E50" s="15" t="n"/>
+      <c r="C50" s="21" t="n"/>
+      <c r="D50" s="21" t="n"/>
+      <c r="E50" s="28">
+        <f>IF(OR(C50="",D50=""),"",MOD(D50-C50,1))</f>
+        <v/>
+      </c>
       <c r="F50" s="15" t="n"/>
       <c r="G50" s="15" t="n"/>
       <c r="H50" s="15" t="n"/>
@@ -2886,16 +3239,22 @@
       <c r="Z50" s="15" t="n"/>
       <c r="AA50" s="15" t="n"/>
       <c r="AB50" s="15" t="n"/>
-      <c r="AC50" s="3" t="n"/>
-      <c r="AD50" s="3" t="n"/>
+      <c r="AC50" s="15" t="n"/>
+      <c r="AD50" s="15" t="n"/>
+      <c r="AE50" s="15" t="n"/>
+      <c r="AF50" s="3" t="n"/>
+      <c r="AG50" s="3" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="24" t="n">
+      <c r="B51" s="27" t="n">
         <v>46338</v>
       </c>
-      <c r="C51" s="15" t="n"/>
-      <c r="D51" s="15" t="n"/>
-      <c r="E51" s="15" t="n"/>
+      <c r="C51" s="21" t="n"/>
+      <c r="D51" s="21" t="n"/>
+      <c r="E51" s="28">
+        <f>IF(OR(C51="",D51=""),"",MOD(D51-C51,1))</f>
+        <v/>
+      </c>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n"/>
       <c r="H51" s="15" t="n"/>
@@ -2919,16 +3278,22 @@
       <c r="Z51" s="15" t="n"/>
       <c r="AA51" s="15" t="n"/>
       <c r="AB51" s="15" t="n"/>
-      <c r="AC51" s="3" t="n"/>
-      <c r="AD51" s="3" t="n"/>
+      <c r="AC51" s="15" t="n"/>
+      <c r="AD51" s="15" t="n"/>
+      <c r="AE51" s="15" t="n"/>
+      <c r="AF51" s="3" t="n"/>
+      <c r="AG51" s="3" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="24" t="n">
+      <c r="B52" s="27" t="n">
         <v>46339</v>
       </c>
-      <c r="C52" s="15" t="n"/>
-      <c r="D52" s="15" t="n"/>
-      <c r="E52" s="15" t="n"/>
+      <c r="C52" s="21" t="n"/>
+      <c r="D52" s="21" t="n"/>
+      <c r="E52" s="28">
+        <f>IF(OR(C52="",D52=""),"",MOD(D52-C52,1))</f>
+        <v/>
+      </c>
       <c r="F52" s="15" t="n"/>
       <c r="G52" s="15" t="n"/>
       <c r="H52" s="15" t="n"/>
@@ -2952,16 +3317,22 @@
       <c r="Z52" s="15" t="n"/>
       <c r="AA52" s="15" t="n"/>
       <c r="AB52" s="15" t="n"/>
-      <c r="AC52" s="3" t="n"/>
-      <c r="AD52" s="3" t="n"/>
+      <c r="AC52" s="15" t="n"/>
+      <c r="AD52" s="15" t="n"/>
+      <c r="AE52" s="15" t="n"/>
+      <c r="AF52" s="3" t="n"/>
+      <c r="AG52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="24" t="n">
+      <c r="B53" s="27" t="n">
         <v>46340</v>
       </c>
-      <c r="C53" s="15" t="n"/>
-      <c r="D53" s="15" t="n"/>
-      <c r="E53" s="15" t="n"/>
+      <c r="C53" s="21" t="n"/>
+      <c r="D53" s="21" t="n"/>
+      <c r="E53" s="28">
+        <f>IF(OR(C53="",D53=""),"",MOD(D53-C53,1))</f>
+        <v/>
+      </c>
       <c r="F53" s="15" t="n"/>
       <c r="G53" s="15" t="n"/>
       <c r="H53" s="15" t="n"/>
@@ -2985,16 +3356,22 @@
       <c r="Z53" s="15" t="n"/>
       <c r="AA53" s="15" t="n"/>
       <c r="AB53" s="15" t="n"/>
-      <c r="AC53" s="3" t="n"/>
-      <c r="AD53" s="3" t="n"/>
+      <c r="AC53" s="15" t="n"/>
+      <c r="AD53" s="15" t="n"/>
+      <c r="AE53" s="15" t="n"/>
+      <c r="AF53" s="3" t="n"/>
+      <c r="AG53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="24" t="n">
+      <c r="B54" s="27" t="n">
         <v>46341</v>
       </c>
-      <c r="C54" s="15" t="n"/>
-      <c r="D54" s="15" t="n"/>
-      <c r="E54" s="15" t="n"/>
+      <c r="C54" s="21" t="n"/>
+      <c r="D54" s="21" t="n"/>
+      <c r="E54" s="28">
+        <f>IF(OR(C54="",D54=""),"",MOD(D54-C54,1))</f>
+        <v/>
+      </c>
       <c r="F54" s="15" t="n"/>
       <c r="G54" s="15" t="n"/>
       <c r="H54" s="15" t="n"/>
@@ -3018,16 +3395,22 @@
       <c r="Z54" s="15" t="n"/>
       <c r="AA54" s="15" t="n"/>
       <c r="AB54" s="15" t="n"/>
-      <c r="AC54" s="3" t="n"/>
-      <c r="AD54" s="3" t="n"/>
+      <c r="AC54" s="15" t="n"/>
+      <c r="AD54" s="15" t="n"/>
+      <c r="AE54" s="15" t="n"/>
+      <c r="AF54" s="3" t="n"/>
+      <c r="AG54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="24" t="n">
+      <c r="B55" s="27" t="n">
         <v>46342</v>
       </c>
-      <c r="C55" s="15" t="n"/>
-      <c r="D55" s="15" t="n"/>
-      <c r="E55" s="15" t="n"/>
+      <c r="C55" s="21" t="n"/>
+      <c r="D55" s="21" t="n"/>
+      <c r="E55" s="28">
+        <f>IF(OR(C55="",D55=""),"",MOD(D55-C55,1))</f>
+        <v/>
+      </c>
       <c r="F55" s="15" t="n"/>
       <c r="G55" s="15" t="n"/>
       <c r="H55" s="15" t="n"/>
@@ -3051,16 +3434,22 @@
       <c r="Z55" s="15" t="n"/>
       <c r="AA55" s="15" t="n"/>
       <c r="AB55" s="15" t="n"/>
-      <c r="AC55" s="3" t="n"/>
-      <c r="AD55" s="3" t="n"/>
+      <c r="AC55" s="15" t="n"/>
+      <c r="AD55" s="15" t="n"/>
+      <c r="AE55" s="15" t="n"/>
+      <c r="AF55" s="3" t="n"/>
+      <c r="AG55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="24" t="n">
+      <c r="B56" s="27" t="n">
         <v>46343</v>
       </c>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="15" t="n"/>
-      <c r="E56" s="15" t="n"/>
+      <c r="C56" s="21" t="n"/>
+      <c r="D56" s="21" t="n"/>
+      <c r="E56" s="28">
+        <f>IF(OR(C56="",D56=""),"",MOD(D56-C56,1))</f>
+        <v/>
+      </c>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n"/>
       <c r="H56" s="15" t="n"/>
@@ -3084,16 +3473,22 @@
       <c r="Z56" s="15" t="n"/>
       <c r="AA56" s="15" t="n"/>
       <c r="AB56" s="15" t="n"/>
-      <c r="AC56" s="3" t="n"/>
-      <c r="AD56" s="3" t="n"/>
+      <c r="AC56" s="15" t="n"/>
+      <c r="AD56" s="15" t="n"/>
+      <c r="AE56" s="15" t="n"/>
+      <c r="AF56" s="3" t="n"/>
+      <c r="AG56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="24" t="n">
+      <c r="B57" s="27" t="n">
         <v>46344</v>
       </c>
-      <c r="C57" s="15" t="n"/>
-      <c r="D57" s="15" t="n"/>
-      <c r="E57" s="15" t="n"/>
+      <c r="C57" s="21" t="n"/>
+      <c r="D57" s="21" t="n"/>
+      <c r="E57" s="28">
+        <f>IF(OR(C57="",D57=""),"",MOD(D57-C57,1))</f>
+        <v/>
+      </c>
       <c r="F57" s="15" t="n"/>
       <c r="G57" s="15" t="n"/>
       <c r="H57" s="15" t="n"/>
@@ -3117,16 +3512,22 @@
       <c r="Z57" s="15" t="n"/>
       <c r="AA57" s="15" t="n"/>
       <c r="AB57" s="15" t="n"/>
-      <c r="AC57" s="3" t="n"/>
-      <c r="AD57" s="3" t="n"/>
+      <c r="AC57" s="15" t="n"/>
+      <c r="AD57" s="15" t="n"/>
+      <c r="AE57" s="15" t="n"/>
+      <c r="AF57" s="3" t="n"/>
+      <c r="AG57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="24" t="n">
+      <c r="B58" s="27" t="n">
         <v>46345</v>
       </c>
-      <c r="C58" s="15" t="n"/>
-      <c r="D58" s="15" t="n"/>
-      <c r="E58" s="15" t="n"/>
+      <c r="C58" s="21" t="n"/>
+      <c r="D58" s="21" t="n"/>
+      <c r="E58" s="28">
+        <f>IF(OR(C58="",D58=""),"",MOD(D58-C58,1))</f>
+        <v/>
+      </c>
       <c r="F58" s="15" t="n"/>
       <c r="G58" s="15" t="n"/>
       <c r="H58" s="15" t="n"/>
@@ -3150,16 +3551,22 @@
       <c r="Z58" s="15" t="n"/>
       <c r="AA58" s="15" t="n"/>
       <c r="AB58" s="15" t="n"/>
-      <c r="AC58" s="3" t="n"/>
-      <c r="AD58" s="3" t="n"/>
+      <c r="AC58" s="15" t="n"/>
+      <c r="AD58" s="15" t="n"/>
+      <c r="AE58" s="15" t="n"/>
+      <c r="AF58" s="3" t="n"/>
+      <c r="AG58" s="3" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="24" t="n">
+      <c r="B59" s="27" t="n">
         <v>46346</v>
       </c>
-      <c r="C59" s="15" t="n"/>
-      <c r="D59" s="15" t="n"/>
-      <c r="E59" s="15" t="n"/>
+      <c r="C59" s="21" t="n"/>
+      <c r="D59" s="21" t="n"/>
+      <c r="E59" s="28">
+        <f>IF(OR(C59="",D59=""),"",MOD(D59-C59,1))</f>
+        <v/>
+      </c>
       <c r="F59" s="15" t="n"/>
       <c r="G59" s="15" t="n"/>
       <c r="H59" s="15" t="n"/>
@@ -3183,16 +3590,22 @@
       <c r="Z59" s="15" t="n"/>
       <c r="AA59" s="15" t="n"/>
       <c r="AB59" s="15" t="n"/>
-      <c r="AC59" s="3" t="n"/>
-      <c r="AD59" s="3" t="n"/>
+      <c r="AC59" s="15" t="n"/>
+      <c r="AD59" s="15" t="n"/>
+      <c r="AE59" s="15" t="n"/>
+      <c r="AF59" s="3" t="n"/>
+      <c r="AG59" s="3" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="24" t="n">
+      <c r="B60" s="27" t="n">
         <v>46347</v>
       </c>
-      <c r="C60" s="15" t="n"/>
-      <c r="D60" s="15" t="n"/>
-      <c r="E60" s="15" t="n"/>
+      <c r="C60" s="21" t="n"/>
+      <c r="D60" s="21" t="n"/>
+      <c r="E60" s="28">
+        <f>IF(OR(C60="",D60=""),"",MOD(D60-C60,1))</f>
+        <v/>
+      </c>
       <c r="F60" s="15" t="n"/>
       <c r="G60" s="15" t="n"/>
       <c r="H60" s="15" t="n"/>
@@ -3216,16 +3629,22 @@
       <c r="Z60" s="15" t="n"/>
       <c r="AA60" s="15" t="n"/>
       <c r="AB60" s="15" t="n"/>
-      <c r="AC60" s="3" t="n"/>
-      <c r="AD60" s="3" t="n"/>
+      <c r="AC60" s="15" t="n"/>
+      <c r="AD60" s="15" t="n"/>
+      <c r="AE60" s="15" t="n"/>
+      <c r="AF60" s="3" t="n"/>
+      <c r="AG60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="24" t="n">
+      <c r="B61" s="27" t="n">
         <v>46348</v>
       </c>
-      <c r="C61" s="15" t="n"/>
-      <c r="D61" s="15" t="n"/>
-      <c r="E61" s="15" t="n"/>
+      <c r="C61" s="21" t="n"/>
+      <c r="D61" s="21" t="n"/>
+      <c r="E61" s="28">
+        <f>IF(OR(C61="",D61=""),"",MOD(D61-C61,1))</f>
+        <v/>
+      </c>
       <c r="F61" s="15" t="n"/>
       <c r="G61" s="15" t="n"/>
       <c r="H61" s="15" t="n"/>
@@ -3249,16 +3668,22 @@
       <c r="Z61" s="15" t="n"/>
       <c r="AA61" s="15" t="n"/>
       <c r="AB61" s="15" t="n"/>
-      <c r="AC61" s="3" t="n"/>
-      <c r="AD61" s="3" t="n"/>
+      <c r="AC61" s="15" t="n"/>
+      <c r="AD61" s="15" t="n"/>
+      <c r="AE61" s="15" t="n"/>
+      <c r="AF61" s="3" t="n"/>
+      <c r="AG61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="24" t="n">
+      <c r="B62" s="27" t="n">
         <v>46349</v>
       </c>
-      <c r="C62" s="15" t="n"/>
-      <c r="D62" s="15" t="n"/>
-      <c r="E62" s="15" t="n"/>
+      <c r="C62" s="21" t="n"/>
+      <c r="D62" s="21" t="n"/>
+      <c r="E62" s="28">
+        <f>IF(OR(C62="",D62=""),"",MOD(D62-C62,1))</f>
+        <v/>
+      </c>
       <c r="F62" s="15" t="n"/>
       <c r="G62" s="15" t="n"/>
       <c r="H62" s="15" t="n"/>
@@ -3282,16 +3707,22 @@
       <c r="Z62" s="15" t="n"/>
       <c r="AA62" s="15" t="n"/>
       <c r="AB62" s="15" t="n"/>
-      <c r="AC62" s="3" t="n"/>
-      <c r="AD62" s="3" t="n"/>
+      <c r="AC62" s="15" t="n"/>
+      <c r="AD62" s="15" t="n"/>
+      <c r="AE62" s="15" t="n"/>
+      <c r="AF62" s="3" t="n"/>
+      <c r="AG62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="24" t="n">
+      <c r="B63" s="27" t="n">
         <v>46350</v>
       </c>
-      <c r="C63" s="15" t="n"/>
-      <c r="D63" s="15" t="n"/>
-      <c r="E63" s="15" t="n"/>
+      <c r="C63" s="21" t="n"/>
+      <c r="D63" s="21" t="n"/>
+      <c r="E63" s="28">
+        <f>IF(OR(C63="",D63=""),"",MOD(D63-C63,1))</f>
+        <v/>
+      </c>
       <c r="F63" s="15" t="n"/>
       <c r="G63" s="15" t="n"/>
       <c r="H63" s="15" t="n"/>
@@ -3315,16 +3746,22 @@
       <c r="Z63" s="15" t="n"/>
       <c r="AA63" s="15" t="n"/>
       <c r="AB63" s="15" t="n"/>
-      <c r="AC63" s="3" t="n"/>
-      <c r="AD63" s="3" t="n"/>
+      <c r="AC63" s="15" t="n"/>
+      <c r="AD63" s="15" t="n"/>
+      <c r="AE63" s="15" t="n"/>
+      <c r="AF63" s="3" t="n"/>
+      <c r="AG63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="24" t="n">
+      <c r="B64" s="27" t="n">
         <v>46351</v>
       </c>
-      <c r="C64" s="15" t="n"/>
-      <c r="D64" s="15" t="n"/>
-      <c r="E64" s="15" t="n"/>
+      <c r="C64" s="21" t="n"/>
+      <c r="D64" s="21" t="n"/>
+      <c r="E64" s="28">
+        <f>IF(OR(C64="",D64=""),"",MOD(D64-C64,1))</f>
+        <v/>
+      </c>
       <c r="F64" s="15" t="n"/>
       <c r="G64" s="15" t="n"/>
       <c r="H64" s="15" t="n"/>
@@ -3348,16 +3785,22 @@
       <c r="Z64" s="15" t="n"/>
       <c r="AA64" s="15" t="n"/>
       <c r="AB64" s="15" t="n"/>
-      <c r="AC64" s="3" t="n"/>
-      <c r="AD64" s="3" t="n"/>
+      <c r="AC64" s="15" t="n"/>
+      <c r="AD64" s="15" t="n"/>
+      <c r="AE64" s="15" t="n"/>
+      <c r="AF64" s="3" t="n"/>
+      <c r="AG64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="24" t="n">
+      <c r="B65" s="27" t="n">
         <v>46352</v>
       </c>
-      <c r="C65" s="15" t="n"/>
-      <c r="D65" s="15" t="n"/>
-      <c r="E65" s="15" t="n"/>
+      <c r="C65" s="21" t="n"/>
+      <c r="D65" s="21" t="n"/>
+      <c r="E65" s="28">
+        <f>IF(OR(C65="",D65=""),"",MOD(D65-C65,1))</f>
+        <v/>
+      </c>
       <c r="F65" s="15" t="n"/>
       <c r="G65" s="15" t="n"/>
       <c r="H65" s="15" t="n"/>
@@ -3381,16 +3824,22 @@
       <c r="Z65" s="15" t="n"/>
       <c r="AA65" s="15" t="n"/>
       <c r="AB65" s="15" t="n"/>
-      <c r="AC65" s="3" t="n"/>
-      <c r="AD65" s="3" t="n"/>
+      <c r="AC65" s="15" t="n"/>
+      <c r="AD65" s="15" t="n"/>
+      <c r="AE65" s="15" t="n"/>
+      <c r="AF65" s="3" t="n"/>
+      <c r="AG65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="24" t="n">
+      <c r="B66" s="27" t="n">
         <v>46353</v>
       </c>
-      <c r="C66" s="15" t="n"/>
-      <c r="D66" s="15" t="n"/>
-      <c r="E66" s="15" t="n"/>
+      <c r="C66" s="21" t="n"/>
+      <c r="D66" s="21" t="n"/>
+      <c r="E66" s="28">
+        <f>IF(OR(C66="",D66=""),"",MOD(D66-C66,1))</f>
+        <v/>
+      </c>
       <c r="F66" s="15" t="n"/>
       <c r="G66" s="15" t="n"/>
       <c r="H66" s="15" t="n"/>
@@ -3414,16 +3863,22 @@
       <c r="Z66" s="15" t="n"/>
       <c r="AA66" s="15" t="n"/>
       <c r="AB66" s="15" t="n"/>
-      <c r="AC66" s="3" t="n"/>
-      <c r="AD66" s="3" t="n"/>
+      <c r="AC66" s="15" t="n"/>
+      <c r="AD66" s="15" t="n"/>
+      <c r="AE66" s="15" t="n"/>
+      <c r="AF66" s="3" t="n"/>
+      <c r="AG66" s="3" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="24" t="n">
+      <c r="B67" s="27" t="n">
         <v>46354</v>
       </c>
-      <c r="C67" s="15" t="n"/>
-      <c r="D67" s="15" t="n"/>
-      <c r="E67" s="15" t="n"/>
+      <c r="C67" s="21" t="n"/>
+      <c r="D67" s="21" t="n"/>
+      <c r="E67" s="28">
+        <f>IF(OR(C67="",D67=""),"",MOD(D67-C67,1))</f>
+        <v/>
+      </c>
       <c r="F67" s="15" t="n"/>
       <c r="G67" s="15" t="n"/>
       <c r="H67" s="15" t="n"/>
@@ -3447,16 +3902,22 @@
       <c r="Z67" s="15" t="n"/>
       <c r="AA67" s="15" t="n"/>
       <c r="AB67" s="15" t="n"/>
-      <c r="AC67" s="3" t="n"/>
-      <c r="AD67" s="3" t="n"/>
+      <c r="AC67" s="15" t="n"/>
+      <c r="AD67" s="15" t="n"/>
+      <c r="AE67" s="15" t="n"/>
+      <c r="AF67" s="3" t="n"/>
+      <c r="AG67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="24" t="n">
+      <c r="B68" s="27" t="n">
         <v>46355</v>
       </c>
-      <c r="C68" s="15" t="n"/>
-      <c r="D68" s="15" t="n"/>
-      <c r="E68" s="15" t="n"/>
+      <c r="C68" s="21" t="n"/>
+      <c r="D68" s="21" t="n"/>
+      <c r="E68" s="28">
+        <f>IF(OR(C68="",D68=""),"",MOD(D68-C68,1))</f>
+        <v/>
+      </c>
       <c r="F68" s="15" t="n"/>
       <c r="G68" s="15" t="n"/>
       <c r="H68" s="15" t="n"/>
@@ -3480,16 +3941,22 @@
       <c r="Z68" s="15" t="n"/>
       <c r="AA68" s="15" t="n"/>
       <c r="AB68" s="15" t="n"/>
-      <c r="AC68" s="3" t="n"/>
-      <c r="AD68" s="3" t="n"/>
+      <c r="AC68" s="15" t="n"/>
+      <c r="AD68" s="15" t="n"/>
+      <c r="AE68" s="15" t="n"/>
+      <c r="AF68" s="3" t="n"/>
+      <c r="AG68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="24" t="n">
+      <c r="B69" s="27" t="n">
         <v>46356</v>
       </c>
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="15" t="n"/>
-      <c r="E69" s="15" t="n"/>
+      <c r="C69" s="21" t="n"/>
+      <c r="D69" s="21" t="n"/>
+      <c r="E69" s="28">
+        <f>IF(OR(C69="",D69=""),"",MOD(D69-C69,1))</f>
+        <v/>
+      </c>
       <c r="F69" s="15" t="n"/>
       <c r="G69" s="15" t="n"/>
       <c r="H69" s="15" t="n"/>
@@ -3513,8 +3980,33 @@
       <c r="Z69" s="15" t="n"/>
       <c r="AA69" s="15" t="n"/>
       <c r="AB69" s="15" t="n"/>
-      <c r="AC69" s="3" t="n"/>
-      <c r="AD69" s="3" t="n"/>
+      <c r="AC69" s="15" t="n"/>
+      <c r="AD69" s="15" t="n"/>
+      <c r="AE69" s="15" t="n"/>
+      <c r="AF69" s="3" t="n"/>
+      <c r="AG69" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="D71" s="29" t="inlineStr">
+        <is>
+          <t>סה"כ אוקטובר</t>
+        </is>
+      </c>
+      <c r="E71" s="30">
+        <f>SUM(E9:E39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="D72" s="29" t="inlineStr">
+        <is>
+          <t>סה"כ נובמבר</t>
+        </is>
+      </c>
+      <c r="E72" s="30">
+        <f>SUM(E40:E69)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3715,7 +4207,7 @@
       <c r="V4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="n">
+      <c r="A5" s="31" t="n">
         <v>46296</v>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -3741,7 +4233,7 @@
       <c r="V5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="31" t="n">
         <v>46297</v>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -3767,7 +4259,7 @@
       <c r="V6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="n">
+      <c r="A7" s="31" t="n">
         <v>46298</v>
       </c>
       <c r="B7" s="2" t="n"/>
@@ -3793,7 +4285,7 @@
       <c r="V7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="31" t="n">
         <v>46299</v>
       </c>
       <c r="B8" s="2" t="n"/>
@@ -3819,7 +4311,7 @@
       <c r="V8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="n">
+      <c r="A9" s="31" t="n">
         <v>46300</v>
       </c>
       <c r="B9" s="2" t="n"/>
@@ -3845,7 +4337,7 @@
       <c r="V9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="31" t="n">
         <v>46301</v>
       </c>
       <c r="B10" s="2" t="n"/>
@@ -3871,7 +4363,7 @@
       <c r="V10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="n">
+      <c r="A11" s="31" t="n">
         <v>46302</v>
       </c>
       <c r="B11" s="2" t="n"/>
@@ -3897,7 +4389,7 @@
       <c r="V11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="n">
+      <c r="A12" s="31" t="n">
         <v>46303</v>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -3923,7 +4415,7 @@
       <c r="V12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n">
+      <c r="A13" s="31" t="n">
         <v>46304</v>
       </c>
       <c r="B13" s="2" t="n"/>
@@ -3949,7 +4441,7 @@
       <c r="V13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="n">
+      <c r="A14" s="31" t="n">
         <v>46305</v>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -3975,7 +4467,7 @@
       <c r="V14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="n">
+      <c r="A15" s="31" t="n">
         <v>46306</v>
       </c>
       <c r="B15" s="2" t="n"/>
@@ -4001,7 +4493,7 @@
       <c r="V15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="n">
+      <c r="A16" s="31" t="n">
         <v>46307</v>
       </c>
       <c r="B16" s="2" t="n"/>
@@ -4027,7 +4519,7 @@
       <c r="V16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="n">
+      <c r="A17" s="31" t="n">
         <v>46308</v>
       </c>
       <c r="B17" s="2" t="n"/>
@@ -4053,7 +4545,7 @@
       <c r="V17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="n">
+      <c r="A18" s="31" t="n">
         <v>46309</v>
       </c>
       <c r="B18" s="2" t="n"/>
@@ -4079,7 +4571,7 @@
       <c r="V18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="n">
+      <c r="A19" s="31" t="n">
         <v>46310</v>
       </c>
       <c r="B19" s="2" t="n"/>
@@ -4105,7 +4597,7 @@
       <c r="V19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="n">
+      <c r="A20" s="31" t="n">
         <v>46311</v>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -4131,7 +4623,7 @@
       <c r="V20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="n">
+      <c r="A21" s="31" t="n">
         <v>46312</v>
       </c>
       <c r="B21" s="2" t="n"/>
@@ -4157,7 +4649,7 @@
       <c r="V21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="n">
+      <c r="A22" s="31" t="n">
         <v>46313</v>
       </c>
       <c r="B22" s="2" t="n"/>
@@ -4183,7 +4675,7 @@
       <c r="V22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="n">
+      <c r="A23" s="31" t="n">
         <v>46314</v>
       </c>
       <c r="B23" s="2" t="n"/>
@@ -4209,7 +4701,7 @@
       <c r="V23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="n">
+      <c r="A24" s="31" t="n">
         <v>46315</v>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -4235,7 +4727,7 @@
       <c r="V24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="n">
+      <c r="A25" s="31" t="n">
         <v>46316</v>
       </c>
       <c r="B25" s="2" t="n"/>
@@ -4261,7 +4753,7 @@
       <c r="V25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="n">
+      <c r="A26" s="31" t="n">
         <v>46317</v>
       </c>
       <c r="B26" s="2" t="n"/>
@@ -4287,7 +4779,7 @@
       <c r="V26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="25" t="n">
+      <c r="A27" s="31" t="n">
         <v>46318</v>
       </c>
       <c r="B27" s="2" t="n"/>
@@ -4313,7 +4805,7 @@
       <c r="V27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="n">
+      <c r="A28" s="31" t="n">
         <v>46319</v>
       </c>
       <c r="B28" s="2" t="n"/>
@@ -4339,7 +4831,7 @@
       <c r="V28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="n">
+      <c r="A29" s="31" t="n">
         <v>46320</v>
       </c>
       <c r="B29" s="2" t="n"/>
@@ -4365,7 +4857,7 @@
       <c r="V29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="25" t="n">
+      <c r="A30" s="31" t="n">
         <v>46321</v>
       </c>
       <c r="B30" s="2" t="n"/>
@@ -4391,7 +4883,7 @@
       <c r="V30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="n">
+      <c r="A31" s="31" t="n">
         <v>46322</v>
       </c>
       <c r="B31" s="2" t="n"/>
@@ -4417,7 +4909,7 @@
       <c r="V31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="n">
+      <c r="A32" s="31" t="n">
         <v>46323</v>
       </c>
       <c r="B32" s="2" t="n"/>
@@ -4443,7 +4935,7 @@
       <c r="V32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="25" t="n">
+      <c r="A33" s="31" t="n">
         <v>46324</v>
       </c>
       <c r="B33" s="2" t="n"/>
@@ -4469,7 +4961,7 @@
       <c r="V33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="25" t="n">
+      <c r="A34" s="31" t="n">
         <v>46325</v>
       </c>
       <c r="B34" s="2" t="n"/>
@@ -4495,7 +4987,7 @@
       <c r="V34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="25" t="n">
+      <c r="A35" s="31" t="n">
         <v>46326</v>
       </c>
       <c r="B35" s="2" t="n"/>
@@ -4521,7 +5013,7 @@
       <c r="V35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="25" t="n">
+      <c r="A36" s="31" t="n">
         <v>46327</v>
       </c>
       <c r="B36" s="2" t="n"/>
@@ -4547,7 +5039,7 @@
       <c r="V36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="25" t="n">
+      <c r="A37" s="31" t="n">
         <v>46328</v>
       </c>
       <c r="B37" s="2" t="n"/>
@@ -4573,7 +5065,7 @@
       <c r="V37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="25" t="n">
+      <c r="A38" s="31" t="n">
         <v>46329</v>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -4599,7 +5091,7 @@
       <c r="V38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="25" t="n">
+      <c r="A39" s="31" t="n">
         <v>46330</v>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -4625,7 +5117,7 @@
       <c r="V39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="25" t="n">
+      <c r="A40" s="31" t="n">
         <v>46331</v>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -4651,7 +5143,7 @@
       <c r="V40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="25" t="n">
+      <c r="A41" s="31" t="n">
         <v>46332</v>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -4677,7 +5169,7 @@
       <c r="V41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="n">
+      <c r="A42" s="31" t="n">
         <v>46333</v>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -4703,7 +5195,7 @@
       <c r="V42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="25" t="n">
+      <c r="A43" s="31" t="n">
         <v>46334</v>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -4729,7 +5221,7 @@
       <c r="V43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="25" t="n">
+      <c r="A44" s="31" t="n">
         <v>46335</v>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -4755,7 +5247,7 @@
       <c r="V44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="25" t="n">
+      <c r="A45" s="31" t="n">
         <v>46336</v>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -4781,7 +5273,7 @@
       <c r="V45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="25" t="n">
+      <c r="A46" s="31" t="n">
         <v>46337</v>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -4807,7 +5299,7 @@
       <c r="V46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="25" t="n">
+      <c r="A47" s="31" t="n">
         <v>46338</v>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -4833,7 +5325,7 @@
       <c r="V47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="n">
+      <c r="A48" s="31" t="n">
         <v>46339</v>
       </c>
       <c r="B48" s="2" t="n"/>
@@ -4859,7 +5351,7 @@
       <c r="V48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="25" t="n">
+      <c r="A49" s="31" t="n">
         <v>46340</v>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -4885,7 +5377,7 @@
       <c r="V49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="n">
+      <c r="A50" s="31" t="n">
         <v>46341</v>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -4911,7 +5403,7 @@
       <c r="V50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="25" t="n">
+      <c r="A51" s="31" t="n">
         <v>46342</v>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -4937,7 +5429,7 @@
       <c r="V51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="n">
+      <c r="A52" s="31" t="n">
         <v>46343</v>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -4963,7 +5455,7 @@
       <c r="V52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="25" t="n">
+      <c r="A53" s="31" t="n">
         <v>46344</v>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -4989,7 +5481,7 @@
       <c r="V53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="25" t="n">
+      <c r="A54" s="31" t="n">
         <v>46345</v>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -5015,7 +5507,7 @@
       <c r="V54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="25" t="n">
+      <c r="A55" s="31" t="n">
         <v>46346</v>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -5041,7 +5533,7 @@
       <c r="V55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="25" t="n">
+      <c r="A56" s="31" t="n">
         <v>46347</v>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -5067,7 +5559,7 @@
       <c r="V56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="25" t="n">
+      <c r="A57" s="31" t="n">
         <v>46348</v>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -5093,7 +5585,7 @@
       <c r="V57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="25" t="n">
+      <c r="A58" s="31" t="n">
         <v>46349</v>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -5119,7 +5611,7 @@
       <c r="V58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="25" t="n">
+      <c r="A59" s="31" t="n">
         <v>46350</v>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -5145,7 +5637,7 @@
       <c r="V59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="25" t="n">
+      <c r="A60" s="31" t="n">
         <v>46351</v>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -5171,7 +5663,7 @@
       <c r="V60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="25" t="n">
+      <c r="A61" s="31" t="n">
         <v>46352</v>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -5197,7 +5689,7 @@
       <c r="V61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="25" t="n">
+      <c r="A62" s="31" t="n">
         <v>46353</v>
       </c>
       <c r="B62" s="2" t="n"/>
@@ -5223,7 +5715,7 @@
       <c r="V62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="25" t="n">
+      <c r="A63" s="31" t="n">
         <v>46354</v>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -5249,7 +5741,7 @@
       <c r="V63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="25" t="n">
+      <c r="A64" s="31" t="n">
         <v>46355</v>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -5275,7 +5767,7 @@
       <c r="V64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="25" t="n">
+      <c r="A65" s="31" t="n">
         <v>46356</v>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -5496,7 +5988,7 @@
       <c r="W8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="31" t="n">
         <v>46296</v>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -5522,7 +6014,7 @@
       <c r="W9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="31" t="n">
         <v>46297</v>
       </c>
       <c r="C10" s="2" t="n"/>
@@ -5548,7 +6040,7 @@
       <c r="W10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="31" t="n">
         <v>46298</v>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -5574,7 +6066,7 @@
       <c r="W11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="31" t="n">
         <v>46299</v>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -5600,7 +6092,7 @@
       <c r="W12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="31" t="n">
         <v>46300</v>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -5626,7 +6118,7 @@
       <c r="W13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="31" t="n">
         <v>46301</v>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -5652,7 +6144,7 @@
       <c r="W14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="31" t="n">
         <v>46302</v>
       </c>
       <c r="C15" s="2" t="n"/>
@@ -5678,7 +6170,7 @@
       <c r="W15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="31" t="n">
         <v>46303</v>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -5704,7 +6196,7 @@
       <c r="W16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="25" t="n">
+      <c r="B17" s="31" t="n">
         <v>46304</v>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -5730,7 +6222,7 @@
       <c r="W17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="31" t="n">
         <v>46305</v>
       </c>
       <c r="C18" s="2" t="n"/>
@@ -5756,7 +6248,7 @@
       <c r="W18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="31" t="n">
         <v>46306</v>
       </c>
       <c r="C19" s="2" t="n"/>
@@ -5782,7 +6274,7 @@
       <c r="W19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="31" t="n">
         <v>46307</v>
       </c>
       <c r="C20" s="2" t="n"/>
@@ -5808,7 +6300,7 @@
       <c r="W20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="25" t="n">
+      <c r="B21" s="31" t="n">
         <v>46308</v>
       </c>
       <c r="C21" s="2" t="n"/>
@@ -5834,7 +6326,7 @@
       <c r="W21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="25" t="n">
+      <c r="B22" s="31" t="n">
         <v>46309</v>
       </c>
       <c r="C22" s="2" t="n"/>
@@ -5860,7 +6352,7 @@
       <c r="W22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="25" t="n">
+      <c r="B23" s="31" t="n">
         <v>46310</v>
       </c>
       <c r="C23" s="2" t="n"/>
@@ -5886,7 +6378,7 @@
       <c r="W23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="25" t="n">
+      <c r="B24" s="31" t="n">
         <v>46311</v>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -5912,7 +6404,7 @@
       <c r="W24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="31" t="n">
         <v>46312</v>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -5938,7 +6430,7 @@
       <c r="W25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="25" t="n">
+      <c r="B26" s="31" t="n">
         <v>46313</v>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -5964,7 +6456,7 @@
       <c r="W26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="25" t="n">
+      <c r="B27" s="31" t="n">
         <v>46314</v>
       </c>
       <c r="C27" s="2" t="n"/>
@@ -5990,7 +6482,7 @@
       <c r="W27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="25" t="n">
+      <c r="B28" s="31" t="n">
         <v>46315</v>
       </c>
       <c r="C28" s="2" t="n"/>
@@ -6016,7 +6508,7 @@
       <c r="W28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="25" t="n">
+      <c r="B29" s="31" t="n">
         <v>46316</v>
       </c>
       <c r="C29" s="2" t="n"/>
@@ -6042,7 +6534,7 @@
       <c r="W29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="25" t="n">
+      <c r="B30" s="31" t="n">
         <v>46317</v>
       </c>
       <c r="C30" s="2" t="n"/>
@@ -6068,7 +6560,7 @@
       <c r="W30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="25" t="n">
+      <c r="B31" s="31" t="n">
         <v>46318</v>
       </c>
       <c r="C31" s="2" t="n"/>
@@ -6094,7 +6586,7 @@
       <c r="W31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="25" t="n">
+      <c r="B32" s="31" t="n">
         <v>46319</v>
       </c>
       <c r="C32" s="2" t="n"/>
@@ -6120,7 +6612,7 @@
       <c r="W32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="25" t="n">
+      <c r="B33" s="31" t="n">
         <v>46320</v>
       </c>
       <c r="C33" s="2" t="n"/>
@@ -6146,7 +6638,7 @@
       <c r="W33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="25" t="n">
+      <c r="B34" s="31" t="n">
         <v>46321</v>
       </c>
       <c r="C34" s="2" t="n"/>
@@ -6172,7 +6664,7 @@
       <c r="W34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="25" t="n">
+      <c r="B35" s="31" t="n">
         <v>46322</v>
       </c>
       <c r="C35" s="2" t="n"/>
@@ -6198,7 +6690,7 @@
       <c r="W35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="25" t="n">
+      <c r="B36" s="31" t="n">
         <v>46323</v>
       </c>
       <c r="C36" s="2" t="n"/>
@@ -6224,7 +6716,7 @@
       <c r="W36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="25" t="n">
+      <c r="B37" s="31" t="n">
         <v>46324</v>
       </c>
       <c r="C37" s="2" t="n"/>
@@ -6250,7 +6742,7 @@
       <c r="W37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="25" t="n">
+      <c r="B38" s="31" t="n">
         <v>46325</v>
       </c>
       <c r="C38" s="2" t="n"/>
@@ -6276,7 +6768,7 @@
       <c r="W38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="25" t="n">
+      <c r="B39" s="31" t="n">
         <v>46326</v>
       </c>
       <c r="C39" s="2" t="n"/>
@@ -6302,7 +6794,7 @@
       <c r="W39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="25" t="n">
+      <c r="B40" s="31" t="n">
         <v>46327</v>
       </c>
       <c r="C40" s="2" t="n"/>
@@ -6328,7 +6820,7 @@
       <c r="W40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="25" t="n">
+      <c r="B41" s="31" t="n">
         <v>46328</v>
       </c>
       <c r="C41" s="2" t="n"/>
@@ -6354,7 +6846,7 @@
       <c r="W41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="25" t="n">
+      <c r="B42" s="31" t="n">
         <v>46329</v>
       </c>
       <c r="C42" s="2" t="n"/>
@@ -6380,7 +6872,7 @@
       <c r="W42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="25" t="n">
+      <c r="B43" s="31" t="n">
         <v>46330</v>
       </c>
       <c r="C43" s="2" t="n"/>
@@ -6406,7 +6898,7 @@
       <c r="W43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="25" t="n">
+      <c r="B44" s="31" t="n">
         <v>46331</v>
       </c>
       <c r="C44" s="2" t="n"/>
@@ -6432,7 +6924,7 @@
       <c r="W44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="25" t="n">
+      <c r="B45" s="31" t="n">
         <v>46332</v>
       </c>
       <c r="C45" s="2" t="n"/>
@@ -6458,7 +6950,7 @@
       <c r="W45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="25" t="n">
+      <c r="B46" s="31" t="n">
         <v>46333</v>
       </c>
       <c r="C46" s="2" t="n"/>
@@ -6484,7 +6976,7 @@
       <c r="W46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="25" t="n">
+      <c r="B47" s="31" t="n">
         <v>46334</v>
       </c>
       <c r="C47" s="2" t="n"/>
@@ -6510,7 +7002,7 @@
       <c r="W47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="25" t="n">
+      <c r="B48" s="31" t="n">
         <v>46335</v>
       </c>
       <c r="C48" s="2" t="n"/>
@@ -6536,7 +7028,7 @@
       <c r="W48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="25" t="n">
+      <c r="B49" s="31" t="n">
         <v>46336</v>
       </c>
       <c r="C49" s="2" t="n"/>
@@ -6562,7 +7054,7 @@
       <c r="W49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="25" t="n">
+      <c r="B50" s="31" t="n">
         <v>46337</v>
       </c>
       <c r="C50" s="2" t="n"/>
@@ -6588,7 +7080,7 @@
       <c r="W50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="25" t="n">
+      <c r="B51" s="31" t="n">
         <v>46338</v>
       </c>
       <c r="C51" s="2" t="n"/>
@@ -6614,7 +7106,7 @@
       <c r="W51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="25" t="n">
+      <c r="B52" s="31" t="n">
         <v>46339</v>
       </c>
       <c r="C52" s="2" t="n"/>
@@ -6640,7 +7132,7 @@
       <c r="W52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="25" t="n">
+      <c r="B53" s="31" t="n">
         <v>46340</v>
       </c>
       <c r="C53" s="2" t="n"/>
@@ -6666,7 +7158,7 @@
       <c r="W53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="25" t="n">
+      <c r="B54" s="31" t="n">
         <v>46341</v>
       </c>
       <c r="C54" s="2" t="n"/>
@@ -6692,7 +7184,7 @@
       <c r="W54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="25" t="n">
+      <c r="B55" s="31" t="n">
         <v>46342</v>
       </c>
       <c r="C55" s="2" t="n"/>
@@ -6718,7 +7210,7 @@
       <c r="W55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="25" t="n">
+      <c r="B56" s="31" t="n">
         <v>46343</v>
       </c>
       <c r="C56" s="2" t="n"/>
@@ -6744,7 +7236,7 @@
       <c r="W56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="25" t="n">
+      <c r="B57" s="31" t="n">
         <v>46344</v>
       </c>
       <c r="C57" s="2" t="n"/>
@@ -6770,7 +7262,7 @@
       <c r="W57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="25" t="n">
+      <c r="B58" s="31" t="n">
         <v>46345</v>
       </c>
       <c r="C58" s="2" t="n"/>
@@ -6796,7 +7288,7 @@
       <c r="W58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="25" t="n">
+      <c r="B59" s="31" t="n">
         <v>46346</v>
       </c>
       <c r="C59" s="2" t="n"/>
@@ -6822,7 +7314,7 @@
       <c r="W59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="25" t="n">
+      <c r="B60" s="31" t="n">
         <v>46347</v>
       </c>
       <c r="C60" s="2" t="n"/>
@@ -6848,7 +7340,7 @@
       <c r="W60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="25" t="n">
+      <c r="B61" s="31" t="n">
         <v>46348</v>
       </c>
       <c r="C61" s="2" t="n"/>
@@ -6874,7 +7366,7 @@
       <c r="W61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="25" t="n">
+      <c r="B62" s="31" t="n">
         <v>46349</v>
       </c>
       <c r="C62" s="2" t="n"/>
@@ -6900,7 +7392,7 @@
       <c r="W62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="25" t="n">
+      <c r="B63" s="31" t="n">
         <v>46350</v>
       </c>
       <c r="C63" s="2" t="n"/>
@@ -6926,7 +7418,7 @@
       <c r="W63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="25" t="n">
+      <c r="B64" s="31" t="n">
         <v>46351</v>
       </c>
       <c r="C64" s="2" t="n"/>
@@ -6952,7 +7444,7 @@
       <c r="W64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="25" t="n">
+      <c r="B65" s="31" t="n">
         <v>46352</v>
       </c>
       <c r="C65" s="2" t="n"/>
@@ -6978,7 +7470,7 @@
       <c r="W65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="25" t="n">
+      <c r="B66" s="31" t="n">
         <v>46353</v>
       </c>
       <c r="C66" s="2" t="n"/>
@@ -7004,7 +7496,7 @@
       <c r="W66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="25" t="n">
+      <c r="B67" s="31" t="n">
         <v>46354</v>
       </c>
       <c r="C67" s="2" t="n"/>
@@ -7030,7 +7522,7 @@
       <c r="W67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="25" t="n">
+      <c r="B68" s="31" t="n">
         <v>46355</v>
       </c>
       <c r="C68" s="2" t="n"/>
@@ -7056,7 +7548,7 @@
       <c r="W68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="25" t="n">
+      <c r="B69" s="31" t="n">
         <v>46356</v>
       </c>
       <c r="C69" s="2" t="n"/>
@@ -7258,7 +7750,7 @@
       <c r="W6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="32" t="n">
         <v>46296</v>
       </c>
       <c r="C7" s="2" t="n"/>
@@ -7284,7 +7776,7 @@
       <c r="W7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="32" t="n">
         <v>46297</v>
       </c>
       <c r="C8" s="2" t="n"/>
@@ -7310,7 +7802,7 @@
       <c r="W8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="32" t="n">
         <v>46298</v>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -7336,7 +7828,7 @@
       <c r="W9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="32" t="n">
         <v>46299</v>
       </c>
       <c r="C10" s="2" t="n"/>
@@ -7362,7 +7854,7 @@
       <c r="W10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="32" t="n">
         <v>46300</v>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -7388,7 +7880,7 @@
       <c r="W11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="32" t="n">
         <v>46301</v>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -7414,7 +7906,7 @@
       <c r="W12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="32" t="n">
         <v>46302</v>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -7440,7 +7932,7 @@
       <c r="W13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="26" t="n">
+      <c r="B14" s="32" t="n">
         <v>46303</v>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -7466,7 +7958,7 @@
       <c r="W14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="26" t="n">
+      <c r="B15" s="32" t="n">
         <v>46304</v>
       </c>
       <c r="C15" s="2" t="n"/>
@@ -7492,7 +7984,7 @@
       <c r="W15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="26" t="n">
+      <c r="B16" s="32" t="n">
         <v>46305</v>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -7518,7 +8010,7 @@
       <c r="W16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="26" t="n">
+      <c r="B17" s="32" t="n">
         <v>46306</v>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -7544,7 +8036,7 @@
       <c r="W17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="26" t="n">
+      <c r="B18" s="32" t="n">
         <v>46307</v>
       </c>
       <c r="C18" s="2" t="n"/>
@@ -7570,7 +8062,7 @@
       <c r="W18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="32" t="n">
         <v>46308</v>
       </c>
       <c r="C19" s="2" t="n"/>
@@ -7596,7 +8088,7 @@
       <c r="W19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="26" t="n">
+      <c r="B20" s="32" t="n">
         <v>46309</v>
       </c>
       <c r="C20" s="2" t="n"/>
@@ -7622,7 +8114,7 @@
       <c r="W20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="32" t="n">
         <v>46310</v>
       </c>
       <c r="C21" s="2" t="n"/>
@@ -7648,7 +8140,7 @@
       <c r="W21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="32" t="n">
         <v>46311</v>
       </c>
       <c r="C22" s="2" t="n"/>
@@ -7674,7 +8166,7 @@
       <c r="W22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="32" t="n">
         <v>46312</v>
       </c>
       <c r="C23" s="2" t="n"/>
@@ -7700,7 +8192,7 @@
       <c r="W23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="26" t="n">
+      <c r="B24" s="32" t="n">
         <v>46313</v>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -7726,7 +8218,7 @@
       <c r="W24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="26" t="n">
+      <c r="B25" s="32" t="n">
         <v>46314</v>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -7752,7 +8244,7 @@
       <c r="W25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="32" t="n">
         <v>46315</v>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -7778,7 +8270,7 @@
       <c r="W26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="32" t="n">
         <v>46316</v>
       </c>
       <c r="C27" s="2" t="n"/>
@@ -7804,7 +8296,7 @@
       <c r="W27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="32" t="n">
         <v>46317</v>
       </c>
       <c r="C28" s="2" t="n"/>
@@ -7830,7 +8322,7 @@
       <c r="W28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="26" t="n">
+      <c r="B29" s="32" t="n">
         <v>46318</v>
       </c>
       <c r="C29" s="2" t="n"/>
@@ -7856,7 +8348,7 @@
       <c r="W29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="26" t="n">
+      <c r="B30" s="32" t="n">
         <v>46319</v>
       </c>
       <c r="C30" s="2" t="n"/>
@@ -7882,7 +8374,7 @@
       <c r="W30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="26" t="n">
+      <c r="B31" s="32" t="n">
         <v>46320</v>
       </c>
       <c r="C31" s="2" t="n"/>
@@ -7908,7 +8400,7 @@
       <c r="W31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="26" t="n">
+      <c r="B32" s="32" t="n">
         <v>46321</v>
       </c>
       <c r="C32" s="2" t="n"/>
@@ -7934,7 +8426,7 @@
       <c r="W32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="26" t="n">
+      <c r="B33" s="32" t="n">
         <v>46322</v>
       </c>
       <c r="C33" s="2" t="n"/>
@@ -7960,7 +8452,7 @@
       <c r="W33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="26" t="n">
+      <c r="B34" s="32" t="n">
         <v>46323</v>
       </c>
       <c r="C34" s="2" t="n"/>
@@ -7986,7 +8478,7 @@
       <c r="W34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="26" t="n">
+      <c r="B35" s="32" t="n">
         <v>46324</v>
       </c>
       <c r="C35" s="2" t="n"/>
@@ -8012,7 +8504,7 @@
       <c r="W35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="26" t="n">
+      <c r="B36" s="32" t="n">
         <v>46325</v>
       </c>
       <c r="C36" s="2" t="n"/>
@@ -8038,7 +8530,7 @@
       <c r="W36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="26" t="n">
+      <c r="B37" s="32" t="n">
         <v>46326</v>
       </c>
       <c r="C37" s="2" t="n"/>
@@ -8064,7 +8556,7 @@
       <c r="W37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="26" t="n">
+      <c r="B38" s="32" t="n">
         <v>46327</v>
       </c>
       <c r="C38" s="2" t="n"/>
@@ -8090,7 +8582,7 @@
       <c r="W38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="26" t="n">
+      <c r="B39" s="32" t="n">
         <v>46328</v>
       </c>
       <c r="C39" s="2" t="n"/>
@@ -8116,7 +8608,7 @@
       <c r="W39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="26" t="n">
+      <c r="B40" s="32" t="n">
         <v>46329</v>
       </c>
       <c r="C40" s="2" t="n"/>
@@ -8142,7 +8634,7 @@
       <c r="W40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="26" t="n">
+      <c r="B41" s="32" t="n">
         <v>46330</v>
       </c>
       <c r="C41" s="2" t="n"/>
@@ -8168,7 +8660,7 @@
       <c r="W41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="26" t="n">
+      <c r="B42" s="32" t="n">
         <v>46331</v>
       </c>
       <c r="C42" s="2" t="n"/>
@@ -8194,7 +8686,7 @@
       <c r="W42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="26" t="n">
+      <c r="B43" s="32" t="n">
         <v>46332</v>
       </c>
       <c r="C43" s="2" t="n"/>
@@ -8220,7 +8712,7 @@
       <c r="W43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="26" t="n">
+      <c r="B44" s="32" t="n">
         <v>46333</v>
       </c>
       <c r="C44" s="2" t="n"/>
@@ -8246,7 +8738,7 @@
       <c r="W44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="26" t="n">
+      <c r="B45" s="32" t="n">
         <v>46334</v>
       </c>
       <c r="C45" s="2" t="n"/>
@@ -8272,7 +8764,7 @@
       <c r="W45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="26" t="n">
+      <c r="B46" s="32" t="n">
         <v>46335</v>
       </c>
       <c r="C46" s="2" t="n"/>
@@ -8298,7 +8790,7 @@
       <c r="W46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="26" t="n">
+      <c r="B47" s="32" t="n">
         <v>46336</v>
       </c>
       <c r="C47" s="2" t="n"/>
@@ -8324,7 +8816,7 @@
       <c r="W47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="26" t="n">
+      <c r="B48" s="32" t="n">
         <v>46337</v>
       </c>
       <c r="C48" s="2" t="n"/>
@@ -8350,7 +8842,7 @@
       <c r="W48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="26" t="n">
+      <c r="B49" s="32" t="n">
         <v>46338</v>
       </c>
       <c r="C49" s="2" t="n"/>
@@ -8376,7 +8868,7 @@
       <c r="W49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="26" t="n">
+      <c r="B50" s="32" t="n">
         <v>46339</v>
       </c>
       <c r="C50" s="2" t="n"/>
@@ -8402,7 +8894,7 @@
       <c r="W50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="26" t="n">
+      <c r="B51" s="32" t="n">
         <v>46340</v>
       </c>
       <c r="C51" s="2" t="n"/>
@@ -8428,7 +8920,7 @@
       <c r="W51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="26" t="n">
+      <c r="B52" s="32" t="n">
         <v>46341</v>
       </c>
       <c r="C52" s="2" t="n"/>
@@ -8454,7 +8946,7 @@
       <c r="W52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="26" t="n">
+      <c r="B53" s="32" t="n">
         <v>46342</v>
       </c>
       <c r="C53" s="2" t="n"/>
@@ -8480,7 +8972,7 @@
       <c r="W53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="26" t="n">
+      <c r="B54" s="32" t="n">
         <v>46343</v>
       </c>
       <c r="C54" s="2" t="n"/>
@@ -8506,7 +8998,7 @@
       <c r="W54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="26" t="n">
+      <c r="B55" s="32" t="n">
         <v>46344</v>
       </c>
       <c r="C55" s="2" t="n"/>
@@ -8532,7 +9024,7 @@
       <c r="W55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="26" t="n">
+      <c r="B56" s="32" t="n">
         <v>46345</v>
       </c>
       <c r="C56" s="2" t="n"/>
@@ -8558,7 +9050,7 @@
       <c r="W56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="26" t="n">
+      <c r="B57" s="32" t="n">
         <v>46346</v>
       </c>
       <c r="C57" s="2" t="n"/>
@@ -8584,7 +9076,7 @@
       <c r="W57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="26" t="n">
+      <c r="B58" s="32" t="n">
         <v>46347</v>
       </c>
       <c r="C58" s="2" t="n"/>
@@ -8610,7 +9102,7 @@
       <c r="W58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="26" t="n">
+      <c r="B59" s="32" t="n">
         <v>46348</v>
       </c>
       <c r="C59" s="2" t="n"/>
@@ -8636,7 +9128,7 @@
       <c r="W59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="26" t="n">
+      <c r="B60" s="32" t="n">
         <v>46349</v>
       </c>
       <c r="C60" s="2" t="n"/>
@@ -8662,7 +9154,7 @@
       <c r="W60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="26" t="n">
+      <c r="B61" s="32" t="n">
         <v>46350</v>
       </c>
       <c r="C61" s="2" t="n"/>
@@ -8688,7 +9180,7 @@
       <c r="W61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="26" t="n">
+      <c r="B62" s="32" t="n">
         <v>46351</v>
       </c>
       <c r="C62" s="2" t="n"/>
@@ -8714,7 +9206,7 @@
       <c r="W62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="26" t="n">
+      <c r="B63" s="32" t="n">
         <v>46352</v>
       </c>
       <c r="C63" s="2" t="n"/>
@@ -8740,7 +9232,7 @@
       <c r="W63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="26" t="n">
+      <c r="B64" s="32" t="n">
         <v>46353</v>
       </c>
       <c r="C64" s="2" t="n"/>
@@ -8766,7 +9258,7 @@
       <c r="W64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="26" t="n">
+      <c r="B65" s="32" t="n">
         <v>46354</v>
       </c>
       <c r="C65" s="2" t="n"/>
@@ -8792,7 +9284,7 @@
       <c r="W65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="26" t="n">
+      <c r="B66" s="32" t="n">
         <v>46355</v>
       </c>
       <c r="C66" s="2" t="n"/>
@@ -8818,7 +9310,7 @@
       <c r="W66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="26" t="n">
+      <c r="B67" s="32" t="n">
         <v>46356</v>
       </c>
       <c r="C67" s="2" t="n"/>

</xml_diff>